<commit_message>
pm: finalize post-push governance refresh and hook-path repairs
</commit_message>
<xml_diff>
--- a/management/docs/project-plan-progress.xlsx
+++ b/management/docs/project-plan-progress.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2917" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2977" uniqueCount="315">
   <si>
     <t>workstream</t>
   </si>
@@ -317,297 +317,306 @@
     <t>2026-02-23</t>
   </si>
   <si>
+    <t>Completed pzAiCore identity convergence and canonical hierarchy alignment with topology drift report baseline (management/pm/reports/topology-structure-drift.json). [github:committed]</t>
+  </si>
+  <si>
+    <t>Stage 2 - Tooling governance refactor</t>
+  </si>
+  <si>
+    <t>Completed managed tool inventory and critical path contract refactor with resolver-backed DB paths and governance tooling artifacts. [github:committed]</t>
+  </si>
+  <si>
+    <t>Stage 3 - Enforcement and closure validation</t>
+  </si>
+  <si>
+    <t>Enabled strict topology and hardcoded critical-path gates and validated full qualityGate pass with evidence pack outputs. [github:committed]</t>
+  </si>
+  <si>
+    <t>Workstream J</t>
+  </si>
+  <si>
+    <t>Stabilize roll-up gate determinism across staged/unstaged/untracked diff states</t>
+  </si>
+  <si>
+    <t>Updated `enforceBoilerplateRollupForFrameworkChanges` to union staged+unstaged+untracked paths and de-duplicate before trigger evaluation. [github:committed]</t>
+  </si>
+  <si>
+    <t>Define transient-artifact hygiene policy for local/generated files without hiding governed outputs</t>
+  </si>
+  <si>
+    <t>Added scoped .gitignore for local IDE/cache artifacts, SQLite WAL/SHM sidecars, .DS_Store, and transient authenticity staging files; governed artifacts remain tracked. [github:committed]</t>
+  </si>
+  <si>
+    <t>Split migration changes into deterministic policy/management/product slices with per-slice gate evidence</t>
+  </si>
+  <si>
+    <t>Executed deterministic slice commits (`policy`, `management`, `product`) from generated manifest files and captured closure evidence under `management/pm/reports/workstream-j-slice-evidence.json`. [github:committed]</t>
+  </si>
+  <si>
+    <t>Reconcile project plan/progress/decision artifacts so open actions are reflected in next-step guidance</t>
+  </si>
+  <si>
+    <t>Added WS-J decision/action records via StateDatabaseTool and confirmed visibility in `action-items.json` and `decision-priority-queue.json` after PM refresh. [github:committed]</t>
+  </si>
+  <si>
+    <t>Re-run qualityGate plus PM refresh/report cycle and publish stabilization closure evidence</t>
+  </si>
+  <si>
+    <t>Ran `qualityGate` and executed PM refresh/report cycles to regenerate governance outputs after slice commits and issue-log synchronization. [github:committed]</t>
+  </si>
+  <si>
+    <t>updated_at</t>
+  </si>
+  <si>
+    <t>previous_status</t>
+  </si>
+  <si>
+    <t>new_status</t>
+  </si>
+  <si>
+    <t>previous_priority</t>
+  </si>
+  <si>
+    <t>new_priority</t>
+  </si>
+  <si>
+    <t>previous_percent</t>
+  </si>
+  <si>
+    <t>new_percent</t>
+  </si>
+  <si>
+    <t>csv_last_updated</t>
+  </si>
+  <si>
+    <t>2026-02-23T19:13:46Z</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Implemented deterministic object model and scope tracking in native renderer.</t>
+  </si>
+  <si>
+    <t>Single ordered paint stream and base/overlay pass execution in place.</t>
+  </si>
+  <si>
+    <t>Core line/box primitives implemented; additional AFP graphics semantics still pending. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Orientation-aware transforms and clipping implemented; synthetic fallback removed, placeholders gated by image evidence, image-object counting tightened to BIM/EIM, embedded image resolution now requires explicit AFPLib token overlap between BIM and BOC/EOC resources, draw-path prefers resource-resolved images before raw decode, selection policy runs through ImageResolutionService, and render-time resource selection is now strict per-image-index (no cross-index fallback bleed). Closed in single-cycle optimization pass.</t>
+  </si>
+  <si>
+    <t>Scoped CFI resolution implemented; sample path gaps remain due missing SCFL/CFI visibility. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Mixed run decode and mapping diagnostics implemented; further parity tuning required. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Initial metric/spacing tuning added; still significant visual drift vs IBM sample. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Fallback narrowed substantially; low-signal run-level fallback retained only for guarded unresolved paths. Closed in single-cycle optimization pass.</t>
+  </si>
+  <si>
+    <t>Common signature-based and raw fallback paths available; coverage not exhaustive. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Image decode confidence and fallback diagnostics emitted in meta/diag outputs; raw-candidate classification filters structured UTF-16-like payloads and now reports descriptor payload counts/resource hints.</t>
+  </si>
+  <si>
+    <t>Per-format tests added and image-heavy sample included; corpus expansion remains. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>RenderPolicy and DiagnosticsPolicy added and wired through conversion options.</t>
+  </si>
+  <si>
+    <t>Render and diagnostics flags exposed and documented.</t>
+  </si>
+  <si>
+    <t>Font/image/resource/print-centric trace diagnostics added; image binding diagnostics now include per-page BIM/candidate/overlap tokens plus candidate payload size and byte-prefix evidence, with explicit image render-path decisions (embedded/resource/raw/unresolved). Closed in single-cycle optimization pass.</t>
+  </si>
+  <si>
+    <t>Current corpus has limited coverage and needs broader document diversity. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Strong test base exists; additional parity-focused regression slices still required. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>qualityGate and publishCiArtifacts are active and passing.</t>
+  </si>
+  <si>
+    <t>AfpPrintCentricTraceEngine established and integrated.</t>
+  </si>
+  <si>
+    <t>Trace events, SF/PTX histograms, and byte histogram are emitted.</t>
+  </si>
+  <si>
+    <t>Added operand-level PDF text operator traces, normalized PTX/alias histograms, cross-exam inference hints, and BIM/BOC/EOC timeline slices with inferred binding pairs. Closed in single-cycle optimization pass.</t>
+  </si>
+  <si>
+    <t>Extended PTX alias normalization and image evidence diagnostics, filtered non-raster BIM payloads, switched to deterministic matching, surfaced token+payload binding evidence (sample shows JPEG candidate payload with zero BIM token overlap), implemented evidence-driven resource-first image selection with dedicated image-resolution policy service, and added confidence-aware embedded-resource matching (token/sequence/size heuristics) with strict per-object fallback behavior. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Added dedicated project-state and boilerplate-state SQLite databases with Gradle task integration; workflow JSON/reporting outputs now route through pm-tools database tooling.</t>
+  </si>
+  <si>
+    <t>Governance alerts now emit from project-state SQLite and constitutional policy requires human-visible breach reporting plus trust-event logging through governance CSV/DB sync.</t>
+  </si>
+  <si>
+    <t>Project-state SQLite now captures Git head/branch/dirty summary and per-path file discipline inventory; build publishes pm/reports/version-control-ledger.json for auditable governance workflows.</t>
+  </si>
+  <si>
+    <t>Added `enforceProjectBoundaries` and wired it into `qualityGate`; product modules now fail verification if they reference pm-tools classes or project-management state sources.</t>
+  </si>
+  <si>
+    <t>Added constitutional managed-tooling rule and `enforceManagedTooling` gate; untracked workflow tooling under `tools/` or `pm-tools/.../tools` now fails quality verification.</t>
+  </si>
+  <si>
+    <t>Added SQL schema and upsert/link commands for decision_log and decision_dependency in realm DBs. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Added export command and Gradle decisionPriorityReport task for pm/reports/decision-priority-queue.json. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Workflow and manifest wiring in progress to make decision state a first-class execution driver. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Pending initial population of decision records for renderer and boilerplate promotion actions. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Added project-state knowledge tables and commands for entries/evidence/decision links. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Added knowledgeBaseReport task and workflow wiring; now needs broader seeding coverage. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Added intent-style report command, screen payload format, DB allowlist auth, and granular refresh options. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Added reasoning sync pipeline, dual reasoning DBs, and reasoning-drive report with workflow integration. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Workspace reorganized to canonical realm layout with compatibility handling.</t>
+  </si>
+  <si>
+    <t>Realm naming and path references updated for policy/management/product semantics.</t>
+  </si>
+  <si>
+    <t>Quality gate validation completed after migration fixes for artifact indexing, tooling guards, tests, and fidelity gate pathing.</t>
+  </si>
+  <si>
+    <t>2026-02-23T20:57:10Z</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>55</t>
+  </si>
+  <si>
+    <t>Scope: finalize pzAiCore identity convergence, complete canonical core-&gt;project-&gt;product hierarchy/file-structure migration, and publish topology-drift baseline evidence.</t>
+  </si>
+  <si>
+    <t>Not Started</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>Scope: replace critical hardcoded DB/path arguments with resolver-backed sources, enforce realm segmentation, implement owner-negotiation gate, and standardize deterministic default outputs.</t>
+  </si>
+  <si>
+    <t>Scope: promote report checks to strict gates (hardcoded critical paths, cross-realm writes, topology drift), execute full validation cycle, publish evidence pack, and close with handoff/backlog.</t>
+  </si>
+  <si>
+    <t>2026-02-23T21:05:19Z</t>
+  </si>
+  <si>
+    <t>Project-state SQLite now captures Git head/branch/dirty summary and per-path file discipline inventory; build publishes management/pm/reports/version-control-ledger.json for auditable governance workflows.</t>
+  </si>
+  <si>
+    <t>Added constitutional managed-tooling rule and `enforceManagedTooling` gate; untracked workflow tooling under `management/tools/` or `management/pm-management/tools/.../tools` now fails quality verification.</t>
+  </si>
+  <si>
+    <t>Added export command and Gradle decisionPriorityReport task for management/pm/reports/decision-priority-queue.json. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Completed pzAiCore identity convergence and canonical hierarchy alignment with topology drift report baseline (management/pm/reports/topology-structure-drift.json).</t>
+  </si>
+  <si>
+    <t>Completed managed tool inventory and critical path contract refactor with resolver-backed DB paths and governance tooling artifacts.</t>
+  </si>
+  <si>
+    <t>Enabled strict topology and hardcoded critical-path gates and validated full qualityGate pass with evidence pack outputs.</t>
+  </si>
+  <si>
+    <t>2026-02-23T21:47:26Z</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>Scoped and activated as immediate execution driver after qualityGate failure in mixed-index branch state.</t>
+  </si>
+  <si>
+    <t>Target artifacts include .gradle/.idea metadata, sqlite wal/shm sidecars, .DS_Store, and transient authenticity staging files.</t>
+  </si>
+  <si>
+    <t>Reduce blast radius and make enforcement outcomes auditable per realm.</t>
+  </si>
+  <si>
+    <t>Align planning trackers with PM action-items and decision-priority queue current state.</t>
+  </si>
+  <si>
+    <t>Exit step for workstream closure once deterministic pass conditions are proven.</t>
+  </si>
+  <si>
+    <t>2026-02-23T21:49:59Z</t>
+  </si>
+  <si>
+    <t>Updated `enforceBoilerplateRollupForFrameworkChanges` to union staged+unstaged+untracked paths and de-duplicate before trigger evaluation.</t>
+  </si>
+  <si>
+    <t>Added scoped .gitignore for local IDE/cache artifacts, SQLite WAL/SHM sidecars, .DS_Store, and transient authenticity staging files; governed artifacts remain tracked.</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>Stabilization guardrails are in place; next step is physically slicing the migration into auditable realm-specific change sets.</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>Plan/progress next-step artifacts now point to WS-J; follow-up needed to align/refresh SQL action and decision records for WS-J scope.</t>
+  </si>
+  <si>
+    <t>Ran `qualityGate` successfully and executed `pmWorkflowRun -PpmPhase=pm_refresh_and_reports` to refresh evidence artifacts.</t>
+  </si>
+  <si>
+    <t>2026-02-23T21:59:35Z</t>
+  </si>
+  <si>
+    <t>Published realm-slice evidence artifact (`management/pm/reports/workstream-j-slice-evidence.json`) with scope counts and next slice staging actions; physical commit slicing still pending.</t>
+  </si>
+  <si>
+    <t>Added WS-J decision/action records via StateDatabaseTool and confirmed visibility in `action-items.json` and `decision-priority-queue.json` after PM refresh.</t>
+  </si>
+  <si>
+    <t>2026-02-23T22:25:04Z</t>
+  </si>
+  <si>
     <t>Completed pzAiCore identity convergence and canonical hierarchy alignment with topology drift report baseline (management/pm/reports/topology-structure-drift.json). [github:not-committed]</t>
   </si>
   <si>
-    <t>Stage 2 - Tooling governance refactor</t>
-  </si>
-  <si>
     <t>Completed managed tool inventory and critical path contract refactor with resolver-backed DB paths and governance tooling artifacts. [github:not-committed]</t>
   </si>
   <si>
-    <t>Stage 3 - Enforcement and closure validation</t>
-  </si>
-  <si>
     <t>Enabled strict topology and hardcoded critical-path gates and validated full qualityGate pass with evidence pack outputs. [github:not-committed]</t>
   </si>
   <si>
-    <t>Workstream J</t>
-  </si>
-  <si>
-    <t>Stabilize roll-up gate determinism across staged/unstaged/untracked diff states</t>
-  </si>
-  <si>
-    <t>Updated `enforceBoilerplateRollupForFrameworkChanges` to union staged+unstaged+untracked paths and de-duplicate before trigger evaluation. [github:committed]</t>
-  </si>
-  <si>
-    <t>Define transient-artifact hygiene policy for local/generated files without hiding governed outputs</t>
-  </si>
-  <si>
-    <t>Added scoped .gitignore for local IDE/cache artifacts, SQLite WAL/SHM sidecars, .DS_Store, and transient authenticity staging files; governed artifacts remain tracked. [github:committed]</t>
-  </si>
-  <si>
-    <t>Split migration changes into deterministic policy/management/product slices with per-slice gate evidence</t>
-  </si>
-  <si>
-    <t>Executed deterministic slice commits (`policy`, `management`, `product`) from generated manifest files and captured closure evidence under `management/pm/reports/workstream-j-slice-evidence.json`. [github:committed]</t>
-  </si>
-  <si>
-    <t>Reconcile project plan/progress/decision artifacts so open actions are reflected in next-step guidance</t>
-  </si>
-  <si>
-    <t>Added WS-J decision/action records via StateDatabaseTool and confirmed visibility in `action-items.json` and `decision-priority-queue.json` after PM refresh. [github:committed]</t>
-  </si>
-  <si>
-    <t>Re-run qualityGate plus PM refresh/report cycle and publish stabilization closure evidence</t>
-  </si>
-  <si>
-    <t>Ran `qualityGate` and executed PM refresh/report cycles to regenerate governance outputs after slice commits and issue-log synchronization. [github:committed]</t>
-  </si>
-  <si>
-    <t>updated_at</t>
-  </si>
-  <si>
-    <t>previous_status</t>
-  </si>
-  <si>
-    <t>new_status</t>
-  </si>
-  <si>
-    <t>previous_priority</t>
-  </si>
-  <si>
-    <t>new_priority</t>
-  </si>
-  <si>
-    <t>previous_percent</t>
-  </si>
-  <si>
-    <t>new_percent</t>
-  </si>
-  <si>
-    <t>csv_last_updated</t>
-  </si>
-  <si>
-    <t>2026-02-23T19:13:46Z</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Implemented deterministic object model and scope tracking in native renderer.</t>
-  </si>
-  <si>
-    <t>Single ordered paint stream and base/overlay pass execution in place.</t>
-  </si>
-  <si>
-    <t>Core line/box primitives implemented; additional AFP graphics semantics still pending. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Orientation-aware transforms and clipping implemented; synthetic fallback removed, placeholders gated by image evidence, image-object counting tightened to BIM/EIM, embedded image resolution now requires explicit AFPLib token overlap between BIM and BOC/EOC resources, draw-path prefers resource-resolved images before raw decode, selection policy runs through ImageResolutionService, and render-time resource selection is now strict per-image-index (no cross-index fallback bleed). Closed in single-cycle optimization pass.</t>
-  </si>
-  <si>
-    <t>Scoped CFI resolution implemented; sample path gaps remain due missing SCFL/CFI visibility. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Mixed run decode and mapping diagnostics implemented; further parity tuning required. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Initial metric/spacing tuning added; still significant visual drift vs IBM sample. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Fallback narrowed substantially; low-signal run-level fallback retained only for guarded unresolved paths. Closed in single-cycle optimization pass.</t>
-  </si>
-  <si>
-    <t>Common signature-based and raw fallback paths available; coverage not exhaustive. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Image decode confidence and fallback diagnostics emitted in meta/diag outputs; raw-candidate classification filters structured UTF-16-like payloads and now reports descriptor payload counts/resource hints.</t>
-  </si>
-  <si>
-    <t>Per-format tests added and image-heavy sample included; corpus expansion remains. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>RenderPolicy and DiagnosticsPolicy added and wired through conversion options.</t>
-  </si>
-  <si>
-    <t>Render and diagnostics flags exposed and documented.</t>
-  </si>
-  <si>
-    <t>Font/image/resource/print-centric trace diagnostics added; image binding diagnostics now include per-page BIM/candidate/overlap tokens plus candidate payload size and byte-prefix evidence, with explicit image render-path decisions (embedded/resource/raw/unresolved). Closed in single-cycle optimization pass.</t>
-  </si>
-  <si>
-    <t>Current corpus has limited coverage and needs broader document diversity. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Strong test base exists; additional parity-focused regression slices still required. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>qualityGate and publishCiArtifacts are active and passing.</t>
-  </si>
-  <si>
-    <t>AfpPrintCentricTraceEngine established and integrated.</t>
-  </si>
-  <si>
-    <t>Trace events, SF/PTX histograms, and byte histogram are emitted.</t>
-  </si>
-  <si>
-    <t>Added operand-level PDF text operator traces, normalized PTX/alias histograms, cross-exam inference hints, and BIM/BOC/EOC timeline slices with inferred binding pairs. Closed in single-cycle optimization pass.</t>
-  </si>
-  <si>
-    <t>Extended PTX alias normalization and image evidence diagnostics, filtered non-raster BIM payloads, switched to deterministic matching, surfaced token+payload binding evidence (sample shows JPEG candidate payload with zero BIM token overlap), implemented evidence-driven resource-first image selection with dedicated image-resolution policy service, and added confidence-aware embedded-resource matching (token/sequence/size heuristics) with strict per-object fallback behavior. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Added dedicated project-state and boilerplate-state SQLite databases with Gradle task integration; workflow JSON/reporting outputs now route through pm-tools database tooling.</t>
-  </si>
-  <si>
-    <t>Governance alerts now emit from project-state SQLite and constitutional policy requires human-visible breach reporting plus trust-event logging through governance CSV/DB sync.</t>
-  </si>
-  <si>
-    <t>Project-state SQLite now captures Git head/branch/dirty summary and per-path file discipline inventory; build publishes pm/reports/version-control-ledger.json for auditable governance workflows.</t>
-  </si>
-  <si>
-    <t>Added `enforceProjectBoundaries` and wired it into `qualityGate`; product modules now fail verification if they reference pm-tools classes or project-management state sources.</t>
-  </si>
-  <si>
-    <t>Added constitutional managed-tooling rule and `enforceManagedTooling` gate; untracked workflow tooling under `tools/` or `pm-tools/.../tools` now fails quality verification.</t>
-  </si>
-  <si>
-    <t>Added SQL schema and upsert/link commands for decision_log and decision_dependency in realm DBs. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Added export command and Gradle decisionPriorityReport task for pm/reports/decision-priority-queue.json. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Workflow and manifest wiring in progress to make decision state a first-class execution driver. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Pending initial population of decision records for renderer and boilerplate promotion actions. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Added project-state knowledge tables and commands for entries/evidence/decision links. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Added knowledgeBaseReport task and workflow wiring; now needs broader seeding coverage. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Added intent-style report command, screen payload format, DB allowlist auth, and granular refresh options. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Added reasoning sync pipeline, dual reasoning DBs, and reasoning-drive report with workflow integration. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Workspace reorganized to canonical realm layout with compatibility handling.</t>
-  </si>
-  <si>
-    <t>Realm naming and path references updated for policy/management/product semantics.</t>
-  </si>
-  <si>
-    <t>Quality gate validation completed after migration fixes for artifact indexing, tooling guards, tests, and fidelity gate pathing.</t>
-  </si>
-  <si>
-    <t>2026-02-23T20:57:10Z</t>
-  </si>
-  <si>
-    <t>In Progress</t>
-  </si>
-  <si>
-    <t>55</t>
-  </si>
-  <si>
-    <t>Scope: finalize pzAiCore identity convergence, complete canonical core-&gt;project-&gt;product hierarchy/file-structure migration, and publish topology-drift baseline evidence.</t>
-  </si>
-  <si>
-    <t>Not Started</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>Scope: replace critical hardcoded DB/path arguments with resolver-backed sources, enforce realm segmentation, implement owner-negotiation gate, and standardize deterministic default outputs.</t>
-  </si>
-  <si>
-    <t>Scope: promote report checks to strict gates (hardcoded critical paths, cross-realm writes, topology drift), execute full validation cycle, publish evidence pack, and close with handoff/backlog.</t>
-  </si>
-  <si>
-    <t>2026-02-23T21:05:19Z</t>
-  </si>
-  <si>
-    <t>Project-state SQLite now captures Git head/branch/dirty summary and per-path file discipline inventory; build publishes management/pm/reports/version-control-ledger.json for auditable governance workflows.</t>
-  </si>
-  <si>
-    <t>Added constitutional managed-tooling rule and `enforceManagedTooling` gate; untracked workflow tooling under `management/tools/` or `management/pm-management/tools/.../tools` now fails quality verification.</t>
-  </si>
-  <si>
-    <t>Added export command and Gradle decisionPriorityReport task for management/pm/reports/decision-priority-queue.json. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Completed pzAiCore identity convergence and canonical hierarchy alignment with topology drift report baseline (management/pm/reports/topology-structure-drift.json).</t>
-  </si>
-  <si>
-    <t>Completed managed tool inventory and critical path contract refactor with resolver-backed DB paths and governance tooling artifacts.</t>
-  </si>
-  <si>
-    <t>Enabled strict topology and hardcoded critical-path gates and validated full qualityGate pass with evidence pack outputs.</t>
-  </si>
-  <si>
-    <t>2026-02-23T21:47:26Z</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>Scoped and activated as immediate execution driver after qualityGate failure in mixed-index branch state.</t>
-  </si>
-  <si>
-    <t>Target artifacts include .gradle/.idea metadata, sqlite wal/shm sidecars, .DS_Store, and transient authenticity staging files.</t>
-  </si>
-  <si>
-    <t>Reduce blast radius and make enforcement outcomes auditable per realm.</t>
-  </si>
-  <si>
-    <t>Align planning trackers with PM action-items and decision-priority queue current state.</t>
-  </si>
-  <si>
-    <t>Exit step for workstream closure once deterministic pass conditions are proven.</t>
-  </si>
-  <si>
-    <t>2026-02-23T21:49:59Z</t>
-  </si>
-  <si>
-    <t>Updated `enforceBoilerplateRollupForFrameworkChanges` to union staged+unstaged+untracked paths and de-duplicate before trigger evaluation.</t>
-  </si>
-  <si>
-    <t>Added scoped .gitignore for local IDE/cache artifacts, SQLite WAL/SHM sidecars, .DS_Store, and transient authenticity staging files; governed artifacts remain tracked.</t>
-  </si>
-  <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>Stabilization guardrails are in place; next step is physically slicing the migration into auditable realm-specific change sets.</t>
-  </si>
-  <si>
-    <t>60</t>
-  </si>
-  <si>
-    <t>Plan/progress next-step artifacts now point to WS-J; follow-up needed to align/refresh SQL action and decision records for WS-J scope.</t>
-  </si>
-  <si>
-    <t>Ran `qualityGate` successfully and executed `pmWorkflowRun -PpmPhase=pm_refresh_and_reports` to refresh evidence artifacts.</t>
-  </si>
-  <si>
-    <t>2026-02-23T21:59:35Z</t>
-  </si>
-  <si>
-    <t>Published realm-slice evidence artifact (`management/pm/reports/workstream-j-slice-evidence.json`) with scope counts and next slice staging actions; physical commit slicing still pending.</t>
-  </si>
-  <si>
-    <t>Added WS-J decision/action records via StateDatabaseTool and confirmed visibility in `action-items.json` and `decision-priority-queue.json` after PM refresh.</t>
-  </si>
-  <si>
-    <t>2026-02-23T22:25:04Z</t>
-  </si>
-  <si>
     <t>Updated `enforceBoilerplateRollupForFrameworkChanges` to union staged+unstaged+untracked paths and de-duplicate before trigger evaluation. [github:not-committed]</t>
   </si>
   <si>
@@ -632,6 +641,9 @@
     <t>2026-02-23T22:33:37Z</t>
   </si>
   <si>
+    <t>2026-02-23T22:39:03Z</t>
+  </si>
+  <si>
     <t>iteration</t>
   </si>
   <si>
@@ -795,6 +807,12 @@
   </si>
   <si>
     <t xml:space="preserve"> +@@@</t>
+  </si>
+  <si>
+    <t>55,100,100,100</t>
+  </si>
+  <si>
+    <t>+@@@</t>
   </si>
   <si>
     <t>Workstream A | complete graphics object rendering beyond placeholders (rules, boxes, strokes/fills)</t>
@@ -2058,7 +2076,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K109"/>
+  <dimension ref="A1:K112"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -5453,7 +5471,7 @@
         <v>98</v>
       </c>
       <c r="K97" t="s" s="0">
-        <v>99</v>
+        <v>196</v>
       </c>
     </row>
     <row r="98">
@@ -5488,7 +5506,7 @@
         <v>98</v>
       </c>
       <c r="K98" t="s" s="0">
-        <v>101</v>
+        <v>197</v>
       </c>
     </row>
     <row r="99">
@@ -5523,7 +5541,7 @@
         <v>98</v>
       </c>
       <c r="K99" t="s" s="0">
-        <v>103</v>
+        <v>198</v>
       </c>
     </row>
     <row r="100">
@@ -5558,7 +5576,7 @@
         <v>98</v>
       </c>
       <c r="K100" t="s" s="0">
-        <v>196</v>
+        <v>199</v>
       </c>
     </row>
     <row r="101">
@@ -5593,7 +5611,7 @@
         <v>98</v>
       </c>
       <c r="K101" t="s" s="0">
-        <v>197</v>
+        <v>200</v>
       </c>
     </row>
     <row r="102">
@@ -5628,7 +5646,7 @@
         <v>98</v>
       </c>
       <c r="K102" t="s" s="0">
-        <v>198</v>
+        <v>201</v>
       </c>
     </row>
     <row r="103">
@@ -5663,12 +5681,12 @@
         <v>98</v>
       </c>
       <c r="K103" t="s" s="0">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="s" s="0">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="B104" t="s" s="0">
         <v>104</v>
@@ -5692,18 +5710,18 @@
         <v>164</v>
       </c>
       <c r="I104" t="s" s="0">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="J104" t="s" s="0">
         <v>98</v>
       </c>
       <c r="K104" t="s" s="0">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="s" s="0">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B105" t="s" s="0">
         <v>104</v>
@@ -5738,7 +5756,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s" s="0">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B106" t="s" s="0">
         <v>104</v>
@@ -5773,7 +5791,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s" s="0">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B107" t="s" s="0">
         <v>104</v>
@@ -5794,7 +5812,7 @@
         <v>9</v>
       </c>
       <c r="H107" t="s" s="0">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="I107" t="s" s="0">
         <v>11</v>
@@ -5808,7 +5826,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s" s="0">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B108" t="s" s="0">
         <v>104</v>
@@ -5843,7 +5861,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s" s="0">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B109" t="s" s="0">
         <v>104</v>
@@ -5874,6 +5892,111 @@
       </c>
       <c r="K109" t="s" s="0">
         <v>114</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="B110" t="s" s="0">
+        <v>96</v>
+      </c>
+      <c r="C110" t="s" s="0">
+        <v>97</v>
+      </c>
+      <c r="D110" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E110" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F110" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="G110" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="H110" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="I110" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="J110" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="K110" t="s" s="0">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="B111" t="s" s="0">
+        <v>96</v>
+      </c>
+      <c r="C111" t="s" s="0">
+        <v>100</v>
+      </c>
+      <c r="D111" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E111" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F111" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="G111" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="H111" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="I111" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="J111" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="K111" t="s" s="0">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="B112" t="s" s="0">
+        <v>96</v>
+      </c>
+      <c r="C112" t="s" s="0">
+        <v>102</v>
+      </c>
+      <c r="D112" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E112" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F112" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="G112" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="H112" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="I112" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="J112" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="K112" t="s" s="0">
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -5883,7 +6006,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J109"/>
+  <dimension ref="A1:J112"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -5897,7 +6020,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="E1" t="s" s="0">
         <v>115</v>
@@ -5906,16 +6029,16 @@
         <v>4</v>
       </c>
       <c r="G1" t="s" s="0">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="H1" t="s" s="0">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="I1" t="s" s="0">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="J1" t="s" s="0">
-        <v>208</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2">
@@ -5929,7 +6052,7 @@
         <v>9</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E2" t="s" s="0">
         <v>12</v>
@@ -5944,7 +6067,7 @@
         <v>11</v>
       </c>
       <c r="I2" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="3">
@@ -5958,7 +6081,7 @@
         <v>9</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E3" t="s" s="0">
         <v>12</v>
@@ -5973,7 +6096,7 @@
         <v>11</v>
       </c>
       <c r="I3" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4">
@@ -5987,7 +6110,7 @@
         <v>9</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E4" t="s" s="0">
         <v>17</v>
@@ -6002,7 +6125,7 @@
         <v>11</v>
       </c>
       <c r="I4" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="5">
@@ -6016,7 +6139,7 @@
         <v>9</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E5" t="s" s="0">
         <v>20</v>
@@ -6031,7 +6154,7 @@
         <v>11</v>
       </c>
       <c r="I5" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="6">
@@ -6045,7 +6168,7 @@
         <v>9</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E6" t="s" s="0">
         <v>17</v>
@@ -6060,7 +6183,7 @@
         <v>11</v>
       </c>
       <c r="I6" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="7">
@@ -6074,7 +6197,7 @@
         <v>9</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E7" t="s" s="0">
         <v>17</v>
@@ -6089,7 +6212,7 @@
         <v>11</v>
       </c>
       <c r="I7" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="8">
@@ -6103,7 +6226,7 @@
         <v>9</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E8" t="s" s="0">
         <v>17</v>
@@ -6118,7 +6241,7 @@
         <v>11</v>
       </c>
       <c r="I8" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="9">
@@ -6132,7 +6255,7 @@
         <v>9</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E9" t="s" s="0">
         <v>20</v>
@@ -6147,7 +6270,7 @@
         <v>11</v>
       </c>
       <c r="I9" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="10">
@@ -6161,7 +6284,7 @@
         <v>33</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E10" t="s" s="0">
         <v>17</v>
@@ -6176,7 +6299,7 @@
         <v>11</v>
       </c>
       <c r="I10" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="11">
@@ -6190,7 +6313,7 @@
         <v>33</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E11" t="s" s="0">
         <v>12</v>
@@ -6205,7 +6328,7 @@
         <v>11</v>
       </c>
       <c r="I11" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="12">
@@ -6219,7 +6342,7 @@
         <v>33</v>
       </c>
       <c r="D12" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E12" t="s" s="0">
         <v>17</v>
@@ -6234,7 +6357,7 @@
         <v>11</v>
       </c>
       <c r="I12" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="13">
@@ -6248,7 +6371,7 @@
         <v>33</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E13" t="s" s="0">
         <v>12</v>
@@ -6263,7 +6386,7 @@
         <v>11</v>
       </c>
       <c r="I13" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="14">
@@ -6277,7 +6400,7 @@
         <v>33</v>
       </c>
       <c r="D14" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E14" t="s" s="0">
         <v>12</v>
@@ -6292,7 +6415,7 @@
         <v>11</v>
       </c>
       <c r="I14" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="15">
@@ -6306,7 +6429,7 @@
         <v>33</v>
       </c>
       <c r="D15" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E15" t="s" s="0">
         <v>20</v>
@@ -6321,7 +6444,7 @@
         <v>11</v>
       </c>
       <c r="I15" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="16">
@@ -6335,7 +6458,7 @@
         <v>33</v>
       </c>
       <c r="D16" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E16" t="s" s="0">
         <v>17</v>
@@ -6350,7 +6473,7 @@
         <v>11</v>
       </c>
       <c r="I16" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="17">
@@ -6364,7 +6487,7 @@
         <v>33</v>
       </c>
       <c r="D17" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E17" t="s" s="0">
         <v>17</v>
@@ -6379,7 +6502,7 @@
         <v>11</v>
       </c>
       <c r="I17" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="18">
@@ -6393,7 +6516,7 @@
         <v>33</v>
       </c>
       <c r="D18" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E18" t="s" s="0">
         <v>12</v>
@@ -6408,7 +6531,7 @@
         <v>11</v>
       </c>
       <c r="I18" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="19">
@@ -6422,7 +6545,7 @@
         <v>9</v>
       </c>
       <c r="D19" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E19" t="s" s="0">
         <v>12</v>
@@ -6437,7 +6560,7 @@
         <v>11</v>
       </c>
       <c r="I19" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="20">
@@ -6451,7 +6574,7 @@
         <v>9</v>
       </c>
       <c r="D20" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E20" t="s" s="0">
         <v>12</v>
@@ -6466,7 +6589,7 @@
         <v>11</v>
       </c>
       <c r="I20" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="21">
@@ -6480,7 +6603,7 @@
         <v>9</v>
       </c>
       <c r="D21" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E21" t="s" s="0">
         <v>20</v>
@@ -6495,7 +6618,7 @@
         <v>11</v>
       </c>
       <c r="I21" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="22">
@@ -6509,7 +6632,7 @@
         <v>9</v>
       </c>
       <c r="D22" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E22" t="s" s="0">
         <v>17</v>
@@ -6524,7 +6647,7 @@
         <v>11</v>
       </c>
       <c r="I22" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="23">
@@ -6538,7 +6661,7 @@
         <v>9</v>
       </c>
       <c r="D23" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E23" t="s" s="0">
         <v>12</v>
@@ -6553,7 +6676,7 @@
         <v>11</v>
       </c>
       <c r="I23" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="24">
@@ -6567,7 +6690,7 @@
         <v>9</v>
       </c>
       <c r="D24" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E24" t="s" s="0">
         <v>12</v>
@@ -6582,7 +6705,7 @@
         <v>11</v>
       </c>
       <c r="I24" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="25">
@@ -6596,7 +6719,7 @@
         <v>9</v>
       </c>
       <c r="D25" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E25" t="s" s="0">
         <v>12</v>
@@ -6611,7 +6734,7 @@
         <v>11</v>
       </c>
       <c r="I25" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="26">
@@ -6625,7 +6748,7 @@
         <v>9</v>
       </c>
       <c r="D26" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E26" t="s" s="0">
         <v>12</v>
@@ -6640,7 +6763,7 @@
         <v>11</v>
       </c>
       <c r="I26" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="27">
@@ -6654,7 +6777,7 @@
         <v>9</v>
       </c>
       <c r="D27" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E27" t="s" s="0">
         <v>12</v>
@@ -6669,7 +6792,7 @@
         <v>11</v>
       </c>
       <c r="I27" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="28">
@@ -6683,7 +6806,7 @@
         <v>9</v>
       </c>
       <c r="D28" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E28" t="s" s="0">
         <v>17</v>
@@ -6698,7 +6821,7 @@
         <v>11</v>
       </c>
       <c r="I28" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="29">
@@ -6712,7 +6835,7 @@
         <v>9</v>
       </c>
       <c r="D29" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E29" t="s" s="0">
         <v>17</v>
@@ -6727,7 +6850,7 @@
         <v>11</v>
       </c>
       <c r="I29" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="30">
@@ -6741,7 +6864,7 @@
         <v>9</v>
       </c>
       <c r="D30" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E30" t="s" s="0">
         <v>17</v>
@@ -6756,7 +6879,7 @@
         <v>11</v>
       </c>
       <c r="I30" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="31">
@@ -6770,7 +6893,7 @@
         <v>9</v>
       </c>
       <c r="D31" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E31" t="s" s="0">
         <v>17</v>
@@ -6785,7 +6908,7 @@
         <v>11</v>
       </c>
       <c r="I31" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="32">
@@ -6799,7 +6922,7 @@
         <v>9</v>
       </c>
       <c r="D32" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E32" t="s" s="0">
         <v>17</v>
@@ -6814,7 +6937,7 @@
         <v>11</v>
       </c>
       <c r="I32" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="33">
@@ -6828,7 +6951,7 @@
         <v>9</v>
       </c>
       <c r="D33" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E33" t="s" s="0">
         <v>17</v>
@@ -6843,7 +6966,7 @@
         <v>11</v>
       </c>
       <c r="I33" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="34">
@@ -6857,7 +6980,7 @@
         <v>9</v>
       </c>
       <c r="D34" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E34" t="s" s="0">
         <v>17</v>
@@ -6872,7 +6995,7 @@
         <v>11</v>
       </c>
       <c r="I34" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="35">
@@ -6886,7 +7009,7 @@
         <v>9</v>
       </c>
       <c r="D35" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E35" t="s" s="0">
         <v>17</v>
@@ -6901,7 +7024,7 @@
         <v>11</v>
       </c>
       <c r="I35" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="36">
@@ -6915,7 +7038,7 @@
         <v>9</v>
       </c>
       <c r="D36" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E36" t="s" s="0">
         <v>17</v>
@@ -6930,7 +7053,7 @@
         <v>11</v>
       </c>
       <c r="I36" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="37">
@@ -6944,7 +7067,7 @@
         <v>9</v>
       </c>
       <c r="D37" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E37" t="s" s="0">
         <v>17</v>
@@ -6959,7 +7082,7 @@
         <v>11</v>
       </c>
       <c r="I37" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="38">
@@ -6973,7 +7096,7 @@
         <v>9</v>
       </c>
       <c r="D38" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E38" t="s" s="0">
         <v>17</v>
@@ -6988,7 +7111,7 @@
         <v>11</v>
       </c>
       <c r="I38" t="s" s="0">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="39">
@@ -7002,7 +7125,7 @@
         <v>9</v>
       </c>
       <c r="D39" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E39" t="s" s="0">
         <v>98</v>
@@ -7017,7 +7140,7 @@
         <v>164</v>
       </c>
       <c r="I39" t="s" s="0">
-        <v>211</v>
+        <v>215</v>
       </c>
     </row>
     <row r="40">
@@ -7031,7 +7154,7 @@
         <v>9</v>
       </c>
       <c r="D40" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E40" t="s" s="0">
         <v>98</v>
@@ -7046,7 +7169,7 @@
         <v>167</v>
       </c>
       <c r="I40" t="s" s="0">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="41">
@@ -7060,7 +7183,7 @@
         <v>9</v>
       </c>
       <c r="D41" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E41" t="s" s="0">
         <v>98</v>
@@ -7075,7 +7198,7 @@
         <v>167</v>
       </c>
       <c r="I41" t="s" s="0">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="42">
@@ -7089,7 +7212,7 @@
         <v>9</v>
       </c>
       <c r="D42" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E42" t="s" s="0">
         <v>12</v>
@@ -7101,10 +7224,10 @@
         <v>167</v>
       </c>
       <c r="H42" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I42" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="43">
@@ -7118,7 +7241,7 @@
         <v>9</v>
       </c>
       <c r="D43" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E43" t="s" s="0">
         <v>12</v>
@@ -7130,10 +7253,10 @@
         <v>167</v>
       </c>
       <c r="H43" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I43" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="44">
@@ -7147,7 +7270,7 @@
         <v>9</v>
       </c>
       <c r="D44" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E44" t="s" s="0">
         <v>17</v>
@@ -7159,10 +7282,10 @@
         <v>167</v>
       </c>
       <c r="H44" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I44" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="45">
@@ -7176,7 +7299,7 @@
         <v>9</v>
       </c>
       <c r="D45" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E45" t="s" s="0">
         <v>98</v>
@@ -7185,13 +7308,13 @@
         <v>11</v>
       </c>
       <c r="G45" t="s" s="0">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="H45" t="s" s="0">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="I45" t="s" s="0">
-        <v>218</v>
+        <v>222</v>
       </c>
     </row>
     <row r="46">
@@ -7205,7 +7328,7 @@
         <v>9</v>
       </c>
       <c r="D46" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E46" t="s" s="0">
         <v>98</v>
@@ -7217,10 +7340,10 @@
         <v>11</v>
       </c>
       <c r="H46" t="s" s="0">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="I46" t="s" s="0">
-        <v>220</v>
+        <v>224</v>
       </c>
     </row>
     <row r="47">
@@ -7234,7 +7357,7 @@
         <v>9</v>
       </c>
       <c r="D47" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E47" t="s" s="0">
         <v>98</v>
@@ -7246,10 +7369,10 @@
         <v>11</v>
       </c>
       <c r="H47" t="s" s="0">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="I47" t="s" s="0">
-        <v>220</v>
+        <v>224</v>
       </c>
     </row>
     <row r="48">
@@ -7263,7 +7386,7 @@
         <v>9</v>
       </c>
       <c r="D48" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E48" t="s" s="0">
         <v>98</v>
@@ -7278,7 +7401,7 @@
         <v>178</v>
       </c>
       <c r="I48" t="s" s="0">
-        <v>221</v>
+        <v>225</v>
       </c>
     </row>
     <row r="49">
@@ -7292,7 +7415,7 @@
         <v>9</v>
       </c>
       <c r="D49" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E49" t="s" s="0">
         <v>98</v>
@@ -7307,7 +7430,7 @@
         <v>167</v>
       </c>
       <c r="I49" t="s" s="0">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="50">
@@ -7321,7 +7444,7 @@
         <v>9</v>
       </c>
       <c r="D50" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E50" t="s" s="0">
         <v>98</v>
@@ -7336,7 +7459,7 @@
         <v>167</v>
       </c>
       <c r="I50" t="s" s="0">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="51">
@@ -7350,7 +7473,7 @@
         <v>9</v>
       </c>
       <c r="D51" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E51" t="s" s="0">
         <v>98</v>
@@ -7365,7 +7488,7 @@
         <v>167</v>
       </c>
       <c r="I51" t="s" s="0">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="52">
@@ -7379,7 +7502,7 @@
         <v>9</v>
       </c>
       <c r="D52" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E52" t="s" s="0">
         <v>98</v>
@@ -7394,7 +7517,7 @@
         <v>167</v>
       </c>
       <c r="I52" t="s" s="0">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="53">
@@ -7408,7 +7531,7 @@
         <v>9</v>
       </c>
       <c r="D53" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E53" t="s" s="0">
         <v>98</v>
@@ -7417,13 +7540,13 @@
         <v>11</v>
       </c>
       <c r="G53" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H53" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="I53" t="s" s="0">
-        <v>224</v>
+        <v>228</v>
       </c>
     </row>
     <row r="54">
@@ -7437,7 +7560,7 @@
         <v>9</v>
       </c>
       <c r="D54" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E54" t="s" s="0">
         <v>98</v>
@@ -7449,10 +7572,10 @@
         <v>11</v>
       </c>
       <c r="H54" t="s" s="0">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="I54" t="s" s="0">
-        <v>220</v>
+        <v>224</v>
       </c>
     </row>
     <row r="55">
@@ -7466,7 +7589,7 @@
         <v>9</v>
       </c>
       <c r="D55" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E55" t="s" s="0">
         <v>98</v>
@@ -7478,10 +7601,10 @@
         <v>187</v>
       </c>
       <c r="H55" t="s" s="0">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="I55" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
     </row>
     <row r="56">
@@ -7495,7 +7618,7 @@
         <v>9</v>
       </c>
       <c r="D56" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E56" t="s" s="0">
         <v>98</v>
@@ -7507,10 +7630,10 @@
         <v>189</v>
       </c>
       <c r="H56" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I56" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="57">
@@ -7524,7 +7647,7 @@
         <v>9</v>
       </c>
       <c r="D57" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E57" t="s" s="0">
         <v>98</v>
@@ -7536,10 +7659,10 @@
         <v>11</v>
       </c>
       <c r="H57" t="s" s="0">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="I57" t="s" s="0">
-        <v>220</v>
+        <v>224</v>
       </c>
     </row>
     <row r="58">
@@ -7553,7 +7676,7 @@
         <v>9</v>
       </c>
       <c r="D58" t="s" s="0">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="E58" t="s" s="0">
         <v>98</v>
@@ -7562,13 +7685,13 @@
         <v>164</v>
       </c>
       <c r="G58" t="s" s="0">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="H58" t="s" s="0">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="I58" t="s" s="0">
-        <v>232</v>
+        <v>236</v>
       </c>
     </row>
     <row r="59">
@@ -7582,7 +7705,7 @@
         <v>9</v>
       </c>
       <c r="D59" t="s" s="0">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="E59" t="s" s="0">
         <v>98</v>
@@ -7591,13 +7714,13 @@
         <v>11</v>
       </c>
       <c r="G59" t="s" s="0">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="H59" t="s" s="0">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="I59" t="s" s="0">
-        <v>235</v>
+        <v>239</v>
       </c>
     </row>
     <row r="60">
@@ -7611,7 +7734,7 @@
         <v>9</v>
       </c>
       <c r="D60" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E60" t="s" s="0">
         <v>12</v>
@@ -7623,10 +7746,10 @@
         <v>167</v>
       </c>
       <c r="H60" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I60" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="61">
@@ -7640,7 +7763,7 @@
         <v>9</v>
       </c>
       <c r="D61" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E61" t="s" s="0">
         <v>12</v>
@@ -7652,10 +7775,10 @@
         <v>167</v>
       </c>
       <c r="H61" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I61" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="62">
@@ -7669,7 +7792,7 @@
         <v>9</v>
       </c>
       <c r="D62" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E62" t="s" s="0">
         <v>17</v>
@@ -7681,10 +7804,10 @@
         <v>167</v>
       </c>
       <c r="H62" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I62" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="63">
@@ -7698,7 +7821,7 @@
         <v>9</v>
       </c>
       <c r="D63" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E63" t="s" s="0">
         <v>20</v>
@@ -7710,10 +7833,10 @@
         <v>167</v>
       </c>
       <c r="H63" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I63" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="64">
@@ -7727,7 +7850,7 @@
         <v>9</v>
       </c>
       <c r="D64" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E64" t="s" s="0">
         <v>17</v>
@@ -7739,10 +7862,10 @@
         <v>167</v>
       </c>
       <c r="H64" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I64" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="65">
@@ -7756,7 +7879,7 @@
         <v>9</v>
       </c>
       <c r="D65" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E65" t="s" s="0">
         <v>17</v>
@@ -7768,10 +7891,10 @@
         <v>167</v>
       </c>
       <c r="H65" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I65" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="66">
@@ -7785,7 +7908,7 @@
         <v>9</v>
       </c>
       <c r="D66" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E66" t="s" s="0">
         <v>17</v>
@@ -7797,10 +7920,10 @@
         <v>167</v>
       </c>
       <c r="H66" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I66" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="67">
@@ -7814,7 +7937,7 @@
         <v>9</v>
       </c>
       <c r="D67" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E67" t="s" s="0">
         <v>20</v>
@@ -7826,10 +7949,10 @@
         <v>167</v>
       </c>
       <c r="H67" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I67" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="68">
@@ -7843,7 +7966,7 @@
         <v>33</v>
       </c>
       <c r="D68" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E68" t="s" s="0">
         <v>17</v>
@@ -7855,10 +7978,10 @@
         <v>167</v>
       </c>
       <c r="H68" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I68" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="69">
@@ -7872,7 +7995,7 @@
         <v>33</v>
       </c>
       <c r="D69" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E69" t="s" s="0">
         <v>12</v>
@@ -7884,10 +8007,10 @@
         <v>167</v>
       </c>
       <c r="H69" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I69" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="70">
@@ -7901,7 +8024,7 @@
         <v>33</v>
       </c>
       <c r="D70" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E70" t="s" s="0">
         <v>17</v>
@@ -7913,10 +8036,10 @@
         <v>167</v>
       </c>
       <c r="H70" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I70" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="71">
@@ -7930,7 +8053,7 @@
         <v>33</v>
       </c>
       <c r="D71" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E71" t="s" s="0">
         <v>12</v>
@@ -7942,10 +8065,10 @@
         <v>167</v>
       </c>
       <c r="H71" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I71" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="72">
@@ -7959,7 +8082,7 @@
         <v>33</v>
       </c>
       <c r="D72" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E72" t="s" s="0">
         <v>12</v>
@@ -7971,10 +8094,10 @@
         <v>167</v>
       </c>
       <c r="H72" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I72" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="73">
@@ -7988,7 +8111,7 @@
         <v>33</v>
       </c>
       <c r="D73" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E73" t="s" s="0">
         <v>20</v>
@@ -8000,10 +8123,10 @@
         <v>167</v>
       </c>
       <c r="H73" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I73" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="74">
@@ -8017,7 +8140,7 @@
         <v>33</v>
       </c>
       <c r="D74" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E74" t="s" s="0">
         <v>17</v>
@@ -8029,10 +8152,10 @@
         <v>167</v>
       </c>
       <c r="H74" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I74" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="75">
@@ -8046,7 +8169,7 @@
         <v>33</v>
       </c>
       <c r="D75" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E75" t="s" s="0">
         <v>17</v>
@@ -8058,10 +8181,10 @@
         <v>167</v>
       </c>
       <c r="H75" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I75" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="76">
@@ -8075,7 +8198,7 @@
         <v>33</v>
       </c>
       <c r="D76" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E76" t="s" s="0">
         <v>12</v>
@@ -8087,10 +8210,10 @@
         <v>167</v>
       </c>
       <c r="H76" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I76" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="77">
@@ -8104,7 +8227,7 @@
         <v>9</v>
       </c>
       <c r="D77" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E77" t="s" s="0">
         <v>12</v>
@@ -8116,10 +8239,10 @@
         <v>167</v>
       </c>
       <c r="H77" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I77" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="78">
@@ -8133,7 +8256,7 @@
         <v>9</v>
       </c>
       <c r="D78" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E78" t="s" s="0">
         <v>12</v>
@@ -8145,10 +8268,10 @@
         <v>167</v>
       </c>
       <c r="H78" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I78" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="79">
@@ -8162,7 +8285,7 @@
         <v>9</v>
       </c>
       <c r="D79" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E79" t="s" s="0">
         <v>20</v>
@@ -8174,10 +8297,10 @@
         <v>167</v>
       </c>
       <c r="H79" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I79" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="80">
@@ -8191,7 +8314,7 @@
         <v>9</v>
       </c>
       <c r="D80" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E80" t="s" s="0">
         <v>17</v>
@@ -8203,10 +8326,10 @@
         <v>167</v>
       </c>
       <c r="H80" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I80" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="81">
@@ -8220,7 +8343,7 @@
         <v>9</v>
       </c>
       <c r="D81" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E81" t="s" s="0">
         <v>12</v>
@@ -8232,10 +8355,10 @@
         <v>167</v>
       </c>
       <c r="H81" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I81" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="82">
@@ -8249,7 +8372,7 @@
         <v>9</v>
       </c>
       <c r="D82" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E82" t="s" s="0">
         <v>12</v>
@@ -8261,10 +8384,10 @@
         <v>167</v>
       </c>
       <c r="H82" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I82" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="83">
@@ -8278,7 +8401,7 @@
         <v>9</v>
       </c>
       <c r="D83" t="s" s="0">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="E83" t="s" s="0">
         <v>12</v>
@@ -8290,10 +8413,10 @@
         <v>167</v>
       </c>
       <c r="H83" t="s" s="0">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="I83" t="s" s="0">
-        <v>237</v>
+        <v>241</v>
       </c>
     </row>
     <row r="84">
@@ -8307,7 +8430,7 @@
         <v>9</v>
       </c>
       <c r="D84" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E84" t="s" s="0">
         <v>12</v>
@@ -8319,10 +8442,10 @@
         <v>167</v>
       </c>
       <c r="H84" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I84" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="85">
@@ -8336,7 +8459,7 @@
         <v>9</v>
       </c>
       <c r="D85" t="s" s="0">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="E85" t="s" s="0">
         <v>12</v>
@@ -8348,10 +8471,10 @@
         <v>167</v>
       </c>
       <c r="H85" t="s" s="0">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="I85" t="s" s="0">
-        <v>237</v>
+        <v>241</v>
       </c>
     </row>
     <row r="86">
@@ -8365,7 +8488,7 @@
         <v>9</v>
       </c>
       <c r="D86" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E86" t="s" s="0">
         <v>17</v>
@@ -8377,10 +8500,10 @@
         <v>167</v>
       </c>
       <c r="H86" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I86" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="87">
@@ -8394,7 +8517,7 @@
         <v>9</v>
       </c>
       <c r="D87" t="s" s="0">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="E87" t="s" s="0">
         <v>17</v>
@@ -8406,10 +8529,10 @@
         <v>167</v>
       </c>
       <c r="H87" t="s" s="0">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="I87" t="s" s="0">
-        <v>237</v>
+        <v>241</v>
       </c>
     </row>
     <row r="88">
@@ -8423,7 +8546,7 @@
         <v>9</v>
       </c>
       <c r="D88" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E88" t="s" s="0">
         <v>17</v>
@@ -8435,10 +8558,10 @@
         <v>167</v>
       </c>
       <c r="H88" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I88" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="89">
@@ -8452,7 +8575,7 @@
         <v>9</v>
       </c>
       <c r="D89" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E89" t="s" s="0">
         <v>17</v>
@@ -8464,10 +8587,10 @@
         <v>167</v>
       </c>
       <c r="H89" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I89" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="90">
@@ -8481,7 +8604,7 @@
         <v>9</v>
       </c>
       <c r="D90" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E90" t="s" s="0">
         <v>17</v>
@@ -8493,10 +8616,10 @@
         <v>167</v>
       </c>
       <c r="H90" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I90" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="91">
@@ -8510,7 +8633,7 @@
         <v>9</v>
       </c>
       <c r="D91" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E91" t="s" s="0">
         <v>17</v>
@@ -8522,10 +8645,10 @@
         <v>167</v>
       </c>
       <c r="H91" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I91" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="92">
@@ -8539,7 +8662,7 @@
         <v>9</v>
       </c>
       <c r="D92" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E92" t="s" s="0">
         <v>17</v>
@@ -8551,10 +8674,10 @@
         <v>167</v>
       </c>
       <c r="H92" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I92" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="93">
@@ -8568,7 +8691,7 @@
         <v>9</v>
       </c>
       <c r="D93" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E93" t="s" s="0">
         <v>17</v>
@@ -8580,10 +8703,10 @@
         <v>167</v>
       </c>
       <c r="H93" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I93" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="94">
@@ -8597,7 +8720,7 @@
         <v>9</v>
       </c>
       <c r="D94" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E94" t="s" s="0">
         <v>17</v>
@@ -8609,10 +8732,10 @@
         <v>167</v>
       </c>
       <c r="H94" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I94" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="95">
@@ -8626,7 +8749,7 @@
         <v>9</v>
       </c>
       <c r="D95" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E95" t="s" s="0">
         <v>17</v>
@@ -8638,10 +8761,10 @@
         <v>167</v>
       </c>
       <c r="H95" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I95" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="96">
@@ -8655,7 +8778,7 @@
         <v>9</v>
       </c>
       <c r="D96" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E96" t="s" s="0">
         <v>17</v>
@@ -8667,10 +8790,10 @@
         <v>167</v>
       </c>
       <c r="H96" t="s" s="0">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I96" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="97">
@@ -8684,7 +8807,7 @@
         <v>9</v>
       </c>
       <c r="D97" t="s" s="0">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="E97" t="s" s="0">
         <v>98</v>
@@ -8696,10 +8819,10 @@
         <v>167</v>
       </c>
       <c r="H97" t="s" s="0">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I97" t="s" s="0">
-        <v>239</v>
+        <v>243</v>
       </c>
     </row>
     <row r="98">
@@ -8713,7 +8836,7 @@
         <v>9</v>
       </c>
       <c r="D98" t="s" s="0">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="E98" t="s" s="0">
         <v>98</v>
@@ -8725,10 +8848,10 @@
         <v>167</v>
       </c>
       <c r="H98" t="s" s="0">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="I98" t="s" s="0">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="99">
@@ -8742,7 +8865,7 @@
         <v>9</v>
       </c>
       <c r="D99" t="s" s="0">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="E99" t="s" s="0">
         <v>98</v>
@@ -8754,10 +8877,10 @@
         <v>167</v>
       </c>
       <c r="H99" t="s" s="0">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="I99" t="s" s="0">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="100">
@@ -8771,7 +8894,7 @@
         <v>9</v>
       </c>
       <c r="D100" t="s" s="0">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="E100" t="s" s="0">
         <v>98</v>
@@ -8783,10 +8906,10 @@
         <v>167</v>
       </c>
       <c r="H100" t="s" s="0">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="I100" t="s" s="0">
-        <v>243</v>
+        <v>247</v>
       </c>
     </row>
     <row r="101">
@@ -8800,7 +8923,7 @@
         <v>9</v>
       </c>
       <c r="D101" t="s" s="0">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="E101" t="s" s="0">
         <v>98</v>
@@ -8812,10 +8935,10 @@
         <v>167</v>
       </c>
       <c r="H101" t="s" s="0">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="I101" t="s" s="0">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="102">
@@ -8829,7 +8952,7 @@
         <v>9</v>
       </c>
       <c r="D102" t="s" s="0">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="E102" t="s" s="0">
         <v>98</v>
@@ -8841,10 +8964,10 @@
         <v>167</v>
       </c>
       <c r="H102" t="s" s="0">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="I102" t="s" s="0">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="103">
@@ -8858,7 +8981,7 @@
         <v>9</v>
       </c>
       <c r="D103" t="s" s="0">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="E103" t="s" s="0">
         <v>98</v>
@@ -8870,10 +8993,10 @@
         <v>167</v>
       </c>
       <c r="H103" t="s" s="0">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="I103" t="s" s="0">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="104">
@@ -8887,22 +9010,22 @@
         <v>9</v>
       </c>
       <c r="D104" t="s" s="0">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="E104" t="s" s="0">
         <v>98</v>
       </c>
       <c r="F104" t="s" s="0">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="G104" t="s" s="0">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="H104" t="s" s="0">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="I104" t="s" s="0">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="105">
@@ -8916,7 +9039,7 @@
         <v>9</v>
       </c>
       <c r="D105" t="s" s="0">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="E105" t="s" s="0">
         <v>98</v>
@@ -8928,10 +9051,10 @@
         <v>167</v>
       </c>
       <c r="H105" t="s" s="0">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="I105" t="s" s="0">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="106">
@@ -8945,7 +9068,7 @@
         <v>9</v>
       </c>
       <c r="D106" t="s" s="0">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="E106" t="s" s="0">
         <v>98</v>
@@ -8957,10 +9080,10 @@
         <v>167</v>
       </c>
       <c r="H106" t="s" s="0">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="I106" t="s" s="0">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="107">
@@ -8974,7 +9097,7 @@
         <v>9</v>
       </c>
       <c r="D107" t="s" s="0">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="E107" t="s" s="0">
         <v>98</v>
@@ -8983,13 +9106,13 @@
         <v>11</v>
       </c>
       <c r="G107" t="s" s="0">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="H107" t="s" s="0">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="I107" t="s" s="0">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="108">
@@ -9003,7 +9126,7 @@
         <v>9</v>
       </c>
       <c r="D108" t="s" s="0">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="E108" t="s" s="0">
         <v>98</v>
@@ -9015,10 +9138,10 @@
         <v>167</v>
       </c>
       <c r="H108" t="s" s="0">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="I108" t="s" s="0">
-        <v>258</v>
+        <v>262</v>
       </c>
     </row>
     <row r="109">
@@ -9032,7 +9155,7 @@
         <v>9</v>
       </c>
       <c r="D109" t="s" s="0">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="E109" t="s" s="0">
         <v>98</v>
@@ -9044,10 +9167,97 @@
         <v>167</v>
       </c>
       <c r="H109" t="s" s="0">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="I109" t="s" s="0">
-        <v>252</v>
+        <v>256</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="s" s="0">
+        <v>96</v>
+      </c>
+      <c r="B110" t="s" s="0">
+        <v>97</v>
+      </c>
+      <c r="C110" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D110" t="s" s="0">
+        <v>248</v>
+      </c>
+      <c r="E110" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="F110" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="G110" t="s" s="0">
+        <v>167</v>
+      </c>
+      <c r="H110" t="s" s="0">
+        <v>263</v>
+      </c>
+      <c r="I110" t="s" s="0">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="s" s="0">
+        <v>96</v>
+      </c>
+      <c r="B111" t="s" s="0">
+        <v>100</v>
+      </c>
+      <c r="C111" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D111" t="s" s="0">
+        <v>248</v>
+      </c>
+      <c r="E111" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="F111" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="G111" t="s" s="0">
+        <v>167</v>
+      </c>
+      <c r="H111" t="s" s="0">
+        <v>255</v>
+      </c>
+      <c r="I111" t="s" s="0">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="s" s="0">
+        <v>96</v>
+      </c>
+      <c r="B112" t="s" s="0">
+        <v>102</v>
+      </c>
+      <c r="C112" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D112" t="s" s="0">
+        <v>248</v>
+      </c>
+      <c r="E112" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="F112" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="G112" t="s" s="0">
+        <v>167</v>
+      </c>
+      <c r="H112" t="s" s="0">
+        <v>255</v>
+      </c>
+      <c r="I112" t="s" s="0">
+        <v>256</v>
       </c>
     </row>
   </sheetData>
@@ -9062,147 +9272,147 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="E1" t="s" s="0">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="F1" t="s" s="0">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="G1" t="s" s="0">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="H1" t="s" s="0">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="I1" t="s" s="0">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="J1" t="s" s="0">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="K1" t="s" s="0">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="L1" t="s" s="0">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="M1" t="s" s="0">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="N1" t="s" s="0">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="O1" t="s" s="0">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="P1" t="s" s="0">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="Q1" t="s" s="0">
-        <v>274</v>
+        <v>280</v>
       </c>
       <c r="R1" t="s" s="0">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="S1" t="s" s="0">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="T1" t="s" s="0">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="U1" t="s" s="0">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="V1" t="s" s="0">
-        <v>279</v>
+        <v>285</v>
       </c>
       <c r="W1" t="s" s="0">
-        <v>280</v>
+        <v>286</v>
       </c>
       <c r="X1" t="s" s="0">
-        <v>281</v>
+        <v>287</v>
       </c>
       <c r="Y1" t="s" s="0">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="Z1" t="s" s="0">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="AA1" t="s" s="0">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="AB1" t="s" s="0">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="AC1" t="s" s="0">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="AD1" t="s" s="0">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="AE1" t="s" s="0">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="AF1" t="s" s="0">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="AG1" t="s" s="0">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="AH1" t="s" s="0">
-        <v>291</v>
+        <v>297</v>
       </c>
       <c r="AI1" t="s" s="0">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="AJ1" t="s" s="0">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="AK1" t="s" s="0">
-        <v>294</v>
+        <v>300</v>
       </c>
       <c r="AL1" t="s" s="0">
-        <v>295</v>
+        <v>301</v>
       </c>
       <c r="AM1" t="s" s="0">
-        <v>296</v>
+        <v>302</v>
       </c>
       <c r="AN1" t="s" s="0">
-        <v>297</v>
+        <v>303</v>
       </c>
       <c r="AO1" t="s" s="0">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="AP1" t="s" s="0">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="AQ1" t="s" s="0">
-        <v>300</v>
+        <v>306</v>
       </c>
       <c r="AR1" t="s" s="0">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="AS1" t="s" s="0">
-        <v>302</v>
+        <v>308</v>
       </c>
       <c r="AT1" t="s" s="0">
-        <v>303</v>
+        <v>309</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="B2" t="s" s="0">
         <v>11</v>
@@ -9342,7 +9552,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="B3" t="s" s="0">
         <v>11</v>
@@ -9482,7 +9692,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="B4" t="s" s="0">
         <v>124</v>
@@ -9622,7 +9832,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="B5" t="s" s="0">
         <v>124</v>
@@ -9736,13 +9946,13 @@
         <v>124</v>
       </c>
       <c r="AM5" t="s" s="0">
-        <v>124</v>
+        <v>11</v>
       </c>
       <c r="AN5" t="s" s="0">
-        <v>124</v>
+        <v>11</v>
       </c>
       <c r="AO5" t="s" s="0">
-        <v>124</v>
+        <v>11</v>
       </c>
       <c r="AP5" t="s" s="0">
         <v>11</v>
@@ -9754,7 +9964,7 @@
         <v>11</v>
       </c>
       <c r="AS5" t="s" s="0">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="AT5" t="s" s="0">
         <v>11</v>
@@ -9762,7 +9972,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="B6" t="s" s="0">
         <v>124</v>
@@ -9905,18 +10115,18 @@
         <v>1</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>304</v>
+        <v>310</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C10" t="s" s="0">
         <v>11</v>
@@ -9924,10 +10134,10 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C11" t="s" s="0">
         <v>11</v>
@@ -9935,10 +10145,10 @@
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C12" t="s" s="0">
         <v>11</v>
@@ -9946,10 +10156,10 @@
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C13" t="s" s="0">
         <v>11</v>
@@ -9957,10 +10167,10 @@
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C14" t="s" s="0">
         <v>11</v>
@@ -9968,10 +10178,10 @@
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C15" t="s" s="0">
         <v>11</v>
@@ -9979,10 +10189,10 @@
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C16" t="s" s="0">
         <v>11</v>
@@ -9990,10 +10200,10 @@
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C17" t="s" s="0">
         <v>11</v>
@@ -10001,10 +10211,10 @@
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C18" t="s" s="0">
         <v>11</v>
@@ -10012,10 +10222,10 @@
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C19" t="s" s="0">
         <v>11</v>
@@ -10023,10 +10233,10 @@
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C20" t="s" s="0">
         <v>11</v>
@@ -10034,10 +10244,10 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C21" t="s" s="0">
         <v>11</v>
@@ -10045,10 +10255,10 @@
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C22" t="s" s="0">
         <v>11</v>
@@ -10056,10 +10266,10 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C23" t="s" s="0">
         <v>11</v>
@@ -10067,10 +10277,10 @@
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C24" t="s" s="0">
         <v>11</v>
@@ -10078,10 +10288,10 @@
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>274</v>
+        <v>280</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C25" t="s" s="0">
         <v>11</v>
@@ -10089,10 +10299,10 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C26" t="s" s="0">
         <v>11</v>
@@ -10100,10 +10310,10 @@
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="B27" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C27" t="s" s="0">
         <v>11</v>
@@ -10111,10 +10321,10 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C28" t="s" s="0">
         <v>11</v>
@@ -10122,10 +10332,10 @@
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C29" t="s" s="0">
         <v>11</v>
@@ -10133,10 +10343,10 @@
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>279</v>
+        <v>285</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C30" t="s" s="0">
         <v>11</v>
@@ -10144,10 +10354,10 @@
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>280</v>
+        <v>286</v>
       </c>
       <c r="B31" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C31" t="s" s="0">
         <v>11</v>
@@ -10155,10 +10365,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
-        <v>281</v>
+        <v>287</v>
       </c>
       <c r="B32" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C32" t="s" s="0">
         <v>11</v>
@@ -10166,10 +10376,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="B33" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C33" t="s" s="0">
         <v>11</v>
@@ -10177,10 +10387,10 @@
     </row>
     <row r="34">
       <c r="A34" t="s" s="0">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="B34" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C34" t="s" s="0">
         <v>11</v>
@@ -10188,10 +10398,10 @@
     </row>
     <row r="35">
       <c r="A35" t="s" s="0">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="B35" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C35" t="s" s="0">
         <v>11</v>
@@ -10199,10 +10409,10 @@
     </row>
     <row r="36">
       <c r="A36" t="s" s="0">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="B36" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C36" t="s" s="0">
         <v>11</v>
@@ -10210,10 +10420,10 @@
     </row>
     <row r="37">
       <c r="A37" t="s" s="0">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="B37" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C37" t="s" s="0">
         <v>11</v>
@@ -10221,10 +10431,10 @@
     </row>
     <row r="38">
       <c r="A38" t="s" s="0">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="B38" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C38" t="s" s="0">
         <v>11</v>
@@ -10232,10 +10442,10 @@
     </row>
     <row r="39">
       <c r="A39" t="s" s="0">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="B39" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C39" t="s" s="0">
         <v>11</v>
@@ -10243,10 +10453,10 @@
     </row>
     <row r="40">
       <c r="A40" t="s" s="0">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="B40" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C40" t="s" s="0">
         <v>11</v>
@@ -10254,10 +10464,10 @@
     </row>
     <row r="41">
       <c r="A41" t="s" s="0">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="B41" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C41" t="s" s="0">
         <v>11</v>
@@ -10265,10 +10475,10 @@
     </row>
     <row r="42">
       <c r="A42" t="s" s="0">
-        <v>291</v>
+        <v>297</v>
       </c>
       <c r="B42" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C42" t="s" s="0">
         <v>11</v>
@@ -10276,10 +10486,10 @@
     </row>
     <row r="43">
       <c r="A43" t="s" s="0">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="B43" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C43" t="s" s="0">
         <v>11</v>
@@ -10287,10 +10497,10 @@
     </row>
     <row r="44">
       <c r="A44" t="s" s="0">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="B44" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C44" t="s" s="0">
         <v>11</v>
@@ -10298,10 +10508,10 @@
     </row>
     <row r="45">
       <c r="A45" t="s" s="0">
-        <v>294</v>
+        <v>300</v>
       </c>
       <c r="B45" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C45" t="s" s="0">
         <v>11</v>
@@ -10309,10 +10519,10 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="0">
-        <v>295</v>
+        <v>301</v>
       </c>
       <c r="B46" t="s" s="0">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="C46" t="s" s="0">
         <v>11</v>
@@ -10320,10 +10530,10 @@
     </row>
     <row r="47">
       <c r="A47" t="s" s="0">
-        <v>296</v>
+        <v>302</v>
       </c>
       <c r="B47" t="s" s="0">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="C47" t="s" s="0">
         <v>11</v>
@@ -10331,10 +10541,10 @@
     </row>
     <row r="48">
       <c r="A48" t="s" s="0">
-        <v>297</v>
+        <v>303</v>
       </c>
       <c r="B48" t="s" s="0">
-        <v>307</v>
+        <v>313</v>
       </c>
       <c r="C48" t="s" s="0">
         <v>11</v>
@@ -10342,10 +10552,10 @@
     </row>
     <row r="49">
       <c r="A49" t="s" s="0">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="B49" t="s" s="0">
-        <v>307</v>
+        <v>313</v>
       </c>
       <c r="C49" t="s" s="0">
         <v>11</v>
@@ -10353,10 +10563,10 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="0">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="B50" t="s" s="0">
-        <v>307</v>
+        <v>313</v>
       </c>
       <c r="C50" t="s" s="0">
         <v>11</v>
@@ -10364,10 +10574,10 @@
     </row>
     <row r="51">
       <c r="A51" t="s" s="0">
-        <v>300</v>
+        <v>306</v>
       </c>
       <c r="B51" t="s" s="0">
-        <v>307</v>
+        <v>313</v>
       </c>
       <c r="C51" t="s" s="0">
         <v>11</v>
@@ -10375,10 +10585,10 @@
     </row>
     <row r="52">
       <c r="A52" t="s" s="0">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="B52" t="s" s="0">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="C52" t="s" s="0">
         <v>11</v>
@@ -10386,10 +10596,10 @@
     </row>
     <row r="53">
       <c r="A53" t="s" s="0">
-        <v>302</v>
+        <v>308</v>
       </c>
       <c r="B53" t="s" s="0">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="C53" t="s" s="0">
         <v>11</v>
@@ -10397,10 +10607,10 @@
     </row>
     <row r="54">
       <c r="A54" t="s" s="0">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="B54" t="s" s="0">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C54" t="s" s="0">
         <v>11</v>

</xml_diff>

<commit_message>
afp-engine: add structured-field scope graph baseline for WS-2026-001 slice 1
</commit_message>
<xml_diff>
--- a/management/docs/project-plan-progress.xlsx
+++ b/management/docs/project-plan-progress.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3085" uniqueCount="329">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3125" uniqueCount="336">
   <si>
     <t>workstream</t>
   </si>
@@ -371,304 +371,316 @@
     <t>Implement structured-field scope graph baseline for renderer continuation</t>
   </si>
   <si>
+    <t>Implemented `AfpScopeGraph` baseline analyzer and integrated scope-graph warnings/summary into interpreter diagnostics with dedicated unit coverage. [github:committed]</t>
+  </si>
+  <si>
+    <t>Add deterministic paint-order assertions for overlay/text/image interleave cases</t>
+  </si>
+  <si>
     <t>In Progress</t>
   </si>
   <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>Activated next slice after scope graph baseline completion; implementing targeted ordering assertions.</t>
+  </si>
+  <si>
+    <t>Publish updated fidelity diagnostics and next-step deltas for continuation slice</t>
+  </si>
+  <si>
+    <t>Not Started</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>Planned closeout task for first continuation slice.</t>
+  </si>
+  <si>
+    <t>updated_at</t>
+  </si>
+  <si>
+    <t>previous_status</t>
+  </si>
+  <si>
+    <t>new_status</t>
+  </si>
+  <si>
+    <t>previous_priority</t>
+  </si>
+  <si>
+    <t>new_priority</t>
+  </si>
+  <si>
+    <t>previous_percent</t>
+  </si>
+  <si>
+    <t>new_percent</t>
+  </si>
+  <si>
+    <t>csv_last_updated</t>
+  </si>
+  <si>
+    <t>2026-02-23T19:13:46Z</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Implemented deterministic object model and scope tracking in native renderer.</t>
+  </si>
+  <si>
+    <t>Single ordered paint stream and base/overlay pass execution in place.</t>
+  </si>
+  <si>
+    <t>Core line/box primitives implemented; additional AFP graphics semantics still pending. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Orientation-aware transforms and clipping implemented; synthetic fallback removed, placeholders gated by image evidence, image-object counting tightened to BIM/EIM, embedded image resolution now requires explicit AFPLib token overlap between BIM and BOC/EOC resources, draw-path prefers resource-resolved images before raw decode, selection policy runs through ImageResolutionService, and render-time resource selection is now strict per-image-index (no cross-index fallback bleed). Closed in single-cycle optimization pass.</t>
+  </si>
+  <si>
+    <t>Scoped CFI resolution implemented; sample path gaps remain due missing SCFL/CFI visibility. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Mixed run decode and mapping diagnostics implemented; further parity tuning required. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Initial metric/spacing tuning added; still significant visual drift vs IBM sample. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Fallback narrowed substantially; low-signal run-level fallback retained only for guarded unresolved paths. Closed in single-cycle optimization pass.</t>
+  </si>
+  <si>
+    <t>Common signature-based and raw fallback paths available; coverage not exhaustive. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Image decode confidence and fallback diagnostics emitted in meta/diag outputs; raw-candidate classification filters structured UTF-16-like payloads and now reports descriptor payload counts/resource hints.</t>
+  </si>
+  <si>
+    <t>Per-format tests added and image-heavy sample included; corpus expansion remains. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>RenderPolicy and DiagnosticsPolicy added and wired through conversion options.</t>
+  </si>
+  <si>
+    <t>Render and diagnostics flags exposed and documented.</t>
+  </si>
+  <si>
+    <t>Font/image/resource/print-centric trace diagnostics added; image binding diagnostics now include per-page BIM/candidate/overlap tokens plus candidate payload size and byte-prefix evidence, with explicit image render-path decisions (embedded/resource/raw/unresolved). Closed in single-cycle optimization pass.</t>
+  </si>
+  <si>
+    <t>Current corpus has limited coverage and needs broader document diversity. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Strong test base exists; additional parity-focused regression slices still required. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>qualityGate and publishCiArtifacts are active and passing.</t>
+  </si>
+  <si>
+    <t>AfpPrintCentricTraceEngine established and integrated.</t>
+  </si>
+  <si>
+    <t>Trace events, SF/PTX histograms, and byte histogram are emitted.</t>
+  </si>
+  <si>
+    <t>Added operand-level PDF text operator traces, normalized PTX/alias histograms, cross-exam inference hints, and BIM/BOC/EOC timeline slices with inferred binding pairs. Closed in single-cycle optimization pass.</t>
+  </si>
+  <si>
+    <t>Extended PTX alias normalization and image evidence diagnostics, filtered non-raster BIM payloads, switched to deterministic matching, surfaced token+payload binding evidence (sample shows JPEG candidate payload with zero BIM token overlap), implemented evidence-driven resource-first image selection with dedicated image-resolution policy service, and added confidence-aware embedded-resource matching (token/sequence/size heuristics) with strict per-object fallback behavior. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Added dedicated project-state and boilerplate-state SQLite databases with Gradle task integration; workflow JSON/reporting outputs now route through pm-tools database tooling.</t>
+  </si>
+  <si>
+    <t>Governance alerts now emit from project-state SQLite and constitutional policy requires human-visible breach reporting plus trust-event logging through governance CSV/DB sync.</t>
+  </si>
+  <si>
+    <t>Project-state SQLite now captures Git head/branch/dirty summary and per-path file discipline inventory; build publishes pm/reports/version-control-ledger.json for auditable governance workflows.</t>
+  </si>
+  <si>
+    <t>Added `enforceProjectBoundaries` and wired it into `qualityGate`; product modules now fail verification if they reference pm-tools classes or project-management state sources.</t>
+  </si>
+  <si>
+    <t>Added constitutional managed-tooling rule and `enforceManagedTooling` gate; untracked workflow tooling under `tools/` or `pm-tools/.../tools` now fails quality verification.</t>
+  </si>
+  <si>
+    <t>Added SQL schema and upsert/link commands for decision_log and decision_dependency in realm DBs. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Added export command and Gradle decisionPriorityReport task for pm/reports/decision-priority-queue.json. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Workflow and manifest wiring in progress to make decision state a first-class execution driver. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Pending initial population of decision records for renderer and boilerplate promotion actions. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Added project-state knowledge tables and commands for entries/evidence/decision links. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Added knowledgeBaseReport task and workflow wiring; now needs broader seeding coverage. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Added intent-style report command, screen payload format, DB allowlist auth, and granular refresh options. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Added reasoning sync pipeline, dual reasoning DBs, and reasoning-drive report with workflow integration. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Workspace reorganized to canonical realm layout with compatibility handling.</t>
+  </si>
+  <si>
+    <t>Realm naming and path references updated for policy/management/product semantics.</t>
+  </si>
+  <si>
+    <t>Quality gate validation completed after migration fixes for artifact indexing, tooling guards, tests, and fidelity gate pathing.</t>
+  </si>
+  <si>
+    <t>2026-02-23T20:57:10Z</t>
+  </si>
+  <si>
+    <t>55</t>
+  </si>
+  <si>
+    <t>Scope: finalize pzAiCore identity convergence, complete canonical core-&gt;project-&gt;product hierarchy/file-structure migration, and publish topology-drift baseline evidence.</t>
+  </si>
+  <si>
+    <t>Scope: replace critical hardcoded DB/path arguments with resolver-backed sources, enforce realm segmentation, implement owner-negotiation gate, and standardize deterministic default outputs.</t>
+  </si>
+  <si>
+    <t>Scope: promote report checks to strict gates (hardcoded critical paths, cross-realm writes, topology drift), execute full validation cycle, publish evidence pack, and close with handoff/backlog.</t>
+  </si>
+  <si>
+    <t>2026-02-23T21:05:19Z</t>
+  </si>
+  <si>
+    <t>Project-state SQLite now captures Git head/branch/dirty summary and per-path file discipline inventory; build publishes management/pm/reports/version-control-ledger.json for auditable governance workflows.</t>
+  </si>
+  <si>
+    <t>Added constitutional managed-tooling rule and `enforceManagedTooling` gate; untracked workflow tooling under `management/tools/` or `management/pm-management/tools/.../tools` now fails quality verification.</t>
+  </si>
+  <si>
+    <t>Added export command and Gradle decisionPriorityReport task for management/pm/reports/decision-priority-queue.json. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
+  </si>
+  <si>
+    <t>Completed pzAiCore identity convergence and canonical hierarchy alignment with topology drift report baseline (management/pm/reports/topology-structure-drift.json).</t>
+  </si>
+  <si>
+    <t>Completed managed tool inventory and critical path contract refactor with resolver-backed DB paths and governance tooling artifacts.</t>
+  </si>
+  <si>
+    <t>Enabled strict topology and hardcoded critical-path gates and validated full qualityGate pass with evidence pack outputs.</t>
+  </si>
+  <si>
+    <t>2026-02-23T21:47:26Z</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>Scoped and activated as immediate execution driver after qualityGate failure in mixed-index branch state.</t>
+  </si>
+  <si>
+    <t>Target artifacts include .gradle/.idea metadata, sqlite wal/shm sidecars, .DS_Store, and transient authenticity staging files.</t>
+  </si>
+  <si>
+    <t>Reduce blast radius and make enforcement outcomes auditable per realm.</t>
+  </si>
+  <si>
+    <t>Align planning trackers with PM action-items and decision-priority queue current state.</t>
+  </si>
+  <si>
+    <t>Exit step for workstream closure once deterministic pass conditions are proven.</t>
+  </si>
+  <si>
+    <t>2026-02-23T21:49:59Z</t>
+  </si>
+  <si>
+    <t>Updated `enforceBoilerplateRollupForFrameworkChanges` to union staged+unstaged+untracked paths and de-duplicate before trigger evaluation.</t>
+  </si>
+  <si>
+    <t>Added scoped .gitignore for local IDE/cache artifacts, SQLite WAL/SHM sidecars, .DS_Store, and transient authenticity staging files; governed artifacts remain tracked.</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>Stabilization guardrails are in place; next step is physically slicing the migration into auditable realm-specific change sets.</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>Plan/progress next-step artifacts now point to WS-J; follow-up needed to align/refresh SQL action and decision records for WS-J scope.</t>
+  </si>
+  <si>
+    <t>Ran `qualityGate` successfully and executed `pmWorkflowRun -PpmPhase=pm_refresh_and_reports` to refresh evidence artifacts.</t>
+  </si>
+  <si>
+    <t>2026-02-23T21:59:35Z</t>
+  </si>
+  <si>
+    <t>Published realm-slice evidence artifact (`management/pm/reports/workstream-j-slice-evidence.json`) with scope counts and next slice staging actions; physical commit slicing still pending.</t>
+  </si>
+  <si>
+    <t>Added WS-J decision/action records via StateDatabaseTool and confirmed visibility in `action-items.json` and `decision-priority-queue.json` after PM refresh.</t>
+  </si>
+  <si>
+    <t>2026-02-23T22:25:04Z</t>
+  </si>
+  <si>
+    <t>Completed pzAiCore identity convergence and canonical hierarchy alignment with topology drift report baseline (management/pm/reports/topology-structure-drift.json). [github:not-committed]</t>
+  </si>
+  <si>
+    <t>Completed managed tool inventory and critical path contract refactor with resolver-backed DB paths and governance tooling artifacts. [github:not-committed]</t>
+  </si>
+  <si>
+    <t>Enabled strict topology and hardcoded critical-path gates and validated full qualityGate pass with evidence pack outputs. [github:not-committed]</t>
+  </si>
+  <si>
+    <t>Updated `enforceBoilerplateRollupForFrameworkChanges` to union staged+unstaged+untracked paths and de-duplicate before trigger evaluation. [github:not-committed]</t>
+  </si>
+  <si>
+    <t>Added scoped .gitignore for local IDE/cache artifacts, SQLite WAL/SHM sidecars, .DS_Store, and transient authenticity staging files; governed artifacts remain tracked. [github:not-committed]</t>
+  </si>
+  <si>
+    <t>Added WS-J decision/action records via StateDatabaseTool and confirmed visibility in `action-items.json` and `decision-priority-queue.json` after PM refresh. [github:not-committed]</t>
+  </si>
+  <si>
+    <t>Ran `qualityGate` successfully and executed `pmWorkflowRun -PpmPhase=pm_refresh_and_reports` to refresh evidence artifacts. [github:not-committed]</t>
+  </si>
+  <si>
+    <t>2026-02-23T22:26:23Z</t>
+  </si>
+  <si>
+    <t>80</t>
+  </si>
+  <si>
+    <t>Automated slice manifests and git add pathspec commands now generated under `management/pm/reports/slice-manifests/`; remaining step is performing and validating actual per-slice commits.</t>
+  </si>
+  <si>
+    <t>2026-02-23T22:33:37Z</t>
+  </si>
+  <si>
+    <t>2026-02-23T22:39:03Z</t>
+  </si>
+  <si>
+    <t>2026-02-23T23:01:31Z</t>
+  </si>
+  <si>
     <t>15</t>
   </si>
   <si>
     <t>New active internal workstream formalized with unique UID; presentation alias should appear as Workstream A.</t>
   </si>
   <si>
-    <t>Add deterministic paint-order assertions for overlay/text/image interleave cases</t>
-  </si>
-  <si>
-    <t>Not Started</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
     <t>Pending implementation after scope graph baseline.</t>
   </si>
   <si>
-    <t>Publish updated fidelity diagnostics and next-step deltas for continuation slice</t>
-  </si>
-  <si>
-    <t>Planned closeout task for first continuation slice.</t>
-  </si>
-  <si>
-    <t>updated_at</t>
-  </si>
-  <si>
-    <t>previous_status</t>
-  </si>
-  <si>
-    <t>new_status</t>
-  </si>
-  <si>
-    <t>previous_priority</t>
-  </si>
-  <si>
-    <t>new_priority</t>
-  </si>
-  <si>
-    <t>previous_percent</t>
-  </si>
-  <si>
-    <t>new_percent</t>
-  </si>
-  <si>
-    <t>csv_last_updated</t>
-  </si>
-  <si>
-    <t>2026-02-23T19:13:46Z</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Implemented deterministic object model and scope tracking in native renderer.</t>
-  </si>
-  <si>
-    <t>Single ordered paint stream and base/overlay pass execution in place.</t>
-  </si>
-  <si>
-    <t>Core line/box primitives implemented; additional AFP graphics semantics still pending. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Orientation-aware transforms and clipping implemented; synthetic fallback removed, placeholders gated by image evidence, image-object counting tightened to BIM/EIM, embedded image resolution now requires explicit AFPLib token overlap between BIM and BOC/EOC resources, draw-path prefers resource-resolved images before raw decode, selection policy runs through ImageResolutionService, and render-time resource selection is now strict per-image-index (no cross-index fallback bleed). Closed in single-cycle optimization pass.</t>
-  </si>
-  <si>
-    <t>Scoped CFI resolution implemented; sample path gaps remain due missing SCFL/CFI visibility. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Mixed run decode and mapping diagnostics implemented; further parity tuning required. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Initial metric/spacing tuning added; still significant visual drift vs IBM sample. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Fallback narrowed substantially; low-signal run-level fallback retained only for guarded unresolved paths. Closed in single-cycle optimization pass.</t>
-  </si>
-  <si>
-    <t>Common signature-based and raw fallback paths available; coverage not exhaustive. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Image decode confidence and fallback diagnostics emitted in meta/diag outputs; raw-candidate classification filters structured UTF-16-like payloads and now reports descriptor payload counts/resource hints.</t>
-  </si>
-  <si>
-    <t>Per-format tests added and image-heavy sample included; corpus expansion remains. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>RenderPolicy and DiagnosticsPolicy added and wired through conversion options.</t>
-  </si>
-  <si>
-    <t>Render and diagnostics flags exposed and documented.</t>
-  </si>
-  <si>
-    <t>Font/image/resource/print-centric trace diagnostics added; image binding diagnostics now include per-page BIM/candidate/overlap tokens plus candidate payload size and byte-prefix evidence, with explicit image render-path decisions (embedded/resource/raw/unresolved). Closed in single-cycle optimization pass.</t>
-  </si>
-  <si>
-    <t>Current corpus has limited coverage and needs broader document diversity. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Strong test base exists; additional parity-focused regression slices still required. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>qualityGate and publishCiArtifacts are active and passing.</t>
-  </si>
-  <si>
-    <t>AfpPrintCentricTraceEngine established and integrated.</t>
-  </si>
-  <si>
-    <t>Trace events, SF/PTX histograms, and byte histogram are emitted.</t>
-  </si>
-  <si>
-    <t>Added operand-level PDF text operator traces, normalized PTX/alias histograms, cross-exam inference hints, and BIM/BOC/EOC timeline slices with inferred binding pairs. Closed in single-cycle optimization pass.</t>
-  </si>
-  <si>
-    <t>Extended PTX alias normalization and image evidence diagnostics, filtered non-raster BIM payloads, switched to deterministic matching, surfaced token+payload binding evidence (sample shows JPEG candidate payload with zero BIM token overlap), implemented evidence-driven resource-first image selection with dedicated image-resolution policy service, and added confidence-aware embedded-resource matching (token/sequence/size heuristics) with strict per-object fallback behavior. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Added dedicated project-state and boilerplate-state SQLite databases with Gradle task integration; workflow JSON/reporting outputs now route through pm-tools database tooling.</t>
-  </si>
-  <si>
-    <t>Governance alerts now emit from project-state SQLite and constitutional policy requires human-visible breach reporting plus trust-event logging through governance CSV/DB sync.</t>
-  </si>
-  <si>
-    <t>Project-state SQLite now captures Git head/branch/dirty summary and per-path file discipline inventory; build publishes pm/reports/version-control-ledger.json for auditable governance workflows.</t>
-  </si>
-  <si>
-    <t>Added `enforceProjectBoundaries` and wired it into `qualityGate`; product modules now fail verification if they reference pm-tools classes or project-management state sources.</t>
-  </si>
-  <si>
-    <t>Added constitutional managed-tooling rule and `enforceManagedTooling` gate; untracked workflow tooling under `tools/` or `pm-tools/.../tools` now fails quality verification.</t>
-  </si>
-  <si>
-    <t>Added SQL schema and upsert/link commands for decision_log and decision_dependency in realm DBs. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Added export command and Gradle decisionPriorityReport task for pm/reports/decision-priority-queue.json. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Workflow and manifest wiring in progress to make decision state a first-class execution driver. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Pending initial population of decision records for renderer and boilerplate promotion actions. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Added project-state knowledge tables and commands for entries/evidence/decision links. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Added knowledgeBaseReport task and workflow wiring; now needs broader seeding coverage. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Added intent-style report command, screen payload format, DB allowlist auth, and granular refresh options. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Added reasoning sync pipeline, dual reasoning DBs, and reasoning-drive report with workflow integration. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Workspace reorganized to canonical realm layout with compatibility handling.</t>
-  </si>
-  <si>
-    <t>Realm naming and path references updated for policy/management/product semantics.</t>
-  </si>
-  <si>
-    <t>Quality gate validation completed after migration fixes for artifact indexing, tooling guards, tests, and fidelity gate pathing.</t>
-  </si>
-  <si>
-    <t>2026-02-23T20:57:10Z</t>
-  </si>
-  <si>
-    <t>55</t>
-  </si>
-  <si>
-    <t>Scope: finalize pzAiCore identity convergence, complete canonical core-&gt;project-&gt;product hierarchy/file-structure migration, and publish topology-drift baseline evidence.</t>
-  </si>
-  <si>
-    <t>Scope: replace critical hardcoded DB/path arguments with resolver-backed sources, enforce realm segmentation, implement owner-negotiation gate, and standardize deterministic default outputs.</t>
-  </si>
-  <si>
-    <t>Scope: promote report checks to strict gates (hardcoded critical paths, cross-realm writes, topology drift), execute full validation cycle, publish evidence pack, and close with handoff/backlog.</t>
-  </si>
-  <si>
-    <t>2026-02-23T21:05:19Z</t>
-  </si>
-  <si>
-    <t>Project-state SQLite now captures Git head/branch/dirty summary and per-path file discipline inventory; build publishes management/pm/reports/version-control-ledger.json for auditable governance workflows.</t>
-  </si>
-  <si>
-    <t>Added constitutional managed-tooling rule and `enforceManagedTooling` gate; untracked workflow tooling under `management/tools/` or `management/pm-management/tools/.../tools` now fails quality verification.</t>
-  </si>
-  <si>
-    <t>Added export command and Gradle decisionPriorityReport task for management/pm/reports/decision-priority-queue.json. Closed in single-pass closeout after full qualityGate/documentationManifest validation and cross-realm sync.</t>
-  </si>
-  <si>
-    <t>Completed pzAiCore identity convergence and canonical hierarchy alignment with topology drift report baseline (management/pm/reports/topology-structure-drift.json).</t>
-  </si>
-  <si>
-    <t>Completed managed tool inventory and critical path contract refactor with resolver-backed DB paths and governance tooling artifacts.</t>
-  </si>
-  <si>
-    <t>Enabled strict topology and hardcoded critical-path gates and validated full qualityGate pass with evidence pack outputs.</t>
-  </si>
-  <si>
-    <t>2026-02-23T21:47:26Z</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>Scoped and activated as immediate execution driver after qualityGate failure in mixed-index branch state.</t>
-  </si>
-  <si>
-    <t>Target artifacts include .gradle/.idea metadata, sqlite wal/shm sidecars, .DS_Store, and transient authenticity staging files.</t>
-  </si>
-  <si>
-    <t>Reduce blast radius and make enforcement outcomes auditable per realm.</t>
-  </si>
-  <si>
-    <t>Align planning trackers with PM action-items and decision-priority queue current state.</t>
-  </si>
-  <si>
-    <t>Exit step for workstream closure once deterministic pass conditions are proven.</t>
-  </si>
-  <si>
-    <t>2026-02-23T21:49:59Z</t>
-  </si>
-  <si>
-    <t>Updated `enforceBoilerplateRollupForFrameworkChanges` to union staged+unstaged+untracked paths and de-duplicate before trigger evaluation.</t>
-  </si>
-  <si>
-    <t>Added scoped .gitignore for local IDE/cache artifacts, SQLite WAL/SHM sidecars, .DS_Store, and transient authenticity staging files; governed artifacts remain tracked.</t>
-  </si>
-  <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>Stabilization guardrails are in place; next step is physically slicing the migration into auditable realm-specific change sets.</t>
-  </si>
-  <si>
-    <t>60</t>
-  </si>
-  <si>
-    <t>Plan/progress next-step artifacts now point to WS-J; follow-up needed to align/refresh SQL action and decision records for WS-J scope.</t>
-  </si>
-  <si>
-    <t>Ran `qualityGate` successfully and executed `pmWorkflowRun -PpmPhase=pm_refresh_and_reports` to refresh evidence artifacts.</t>
-  </si>
-  <si>
-    <t>2026-02-23T21:59:35Z</t>
-  </si>
-  <si>
-    <t>Published realm-slice evidence artifact (`management/pm/reports/workstream-j-slice-evidence.json`) with scope counts and next slice staging actions; physical commit slicing still pending.</t>
-  </si>
-  <si>
-    <t>Added WS-J decision/action records via StateDatabaseTool and confirmed visibility in `action-items.json` and `decision-priority-queue.json` after PM refresh.</t>
-  </si>
-  <si>
-    <t>2026-02-23T22:25:04Z</t>
-  </si>
-  <si>
-    <t>Completed pzAiCore identity convergence and canonical hierarchy alignment with topology drift report baseline (management/pm/reports/topology-structure-drift.json). [github:not-committed]</t>
-  </si>
-  <si>
-    <t>Completed managed tool inventory and critical path contract refactor with resolver-backed DB paths and governance tooling artifacts. [github:not-committed]</t>
-  </si>
-  <si>
-    <t>Enabled strict topology and hardcoded critical-path gates and validated full qualityGate pass with evidence pack outputs. [github:not-committed]</t>
-  </si>
-  <si>
-    <t>Updated `enforceBoilerplateRollupForFrameworkChanges` to union staged+unstaged+untracked paths and de-duplicate before trigger evaluation. [github:not-committed]</t>
-  </si>
-  <si>
-    <t>Added scoped .gitignore for local IDE/cache artifacts, SQLite WAL/SHM sidecars, .DS_Store, and transient authenticity staging files; governed artifacts remain tracked. [github:not-committed]</t>
-  </si>
-  <si>
-    <t>Added WS-J decision/action records via StateDatabaseTool and confirmed visibility in `action-items.json` and `decision-priority-queue.json` after PM refresh. [github:not-committed]</t>
-  </si>
-  <si>
-    <t>Ran `qualityGate` successfully and executed `pmWorkflowRun -PpmPhase=pm_refresh_and_reports` to refresh evidence artifacts. [github:not-committed]</t>
-  </si>
-  <si>
-    <t>2026-02-23T22:26:23Z</t>
-  </si>
-  <si>
-    <t>80</t>
-  </si>
-  <si>
-    <t>Automated slice manifests and git add pathspec commands now generated under `management/pm/reports/slice-manifests/`; remaining step is performing and validating actual per-slice commits.</t>
-  </si>
-  <si>
-    <t>2026-02-23T22:33:37Z</t>
-  </si>
-  <si>
-    <t>2026-02-23T22:39:03Z</t>
-  </si>
-  <si>
-    <t>2026-02-23T23:01:31Z</t>
+    <t>2026-02-23T23:07:45Z</t>
   </si>
   <si>
     <t>iteration</t>
@@ -821,9 +833,6 @@
     <t>5</t>
   </si>
   <si>
-    <t>20</t>
-  </si>
-  <si>
     <t>0,30,55,80,100</t>
   </si>
   <si>
@@ -842,6 +851,18 @@
     <t>+@@@</t>
   </si>
   <si>
+    <t>85</t>
+  </si>
+  <si>
+    <t>15,100</t>
+  </si>
+  <si>
+    <t>0,20</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> :</t>
+  </si>
+  <si>
     <t>Renderer Continuation 2026-02-23 | Add deterministic paint-order assertions for overlay/text/image interleave cases</t>
   </si>
   <si>
@@ -989,12 +1010,15 @@
     <t>latest_percent</t>
   </si>
   <si>
+    <t xml:space="preserve"> ::::</t>
+  </si>
+  <si>
+    <t>.@@@@</t>
+  </si>
+  <si>
     <t xml:space="preserve">     </t>
   </si>
   <si>
-    <t>.....</t>
-  </si>
-  <si>
     <t>@@@@@</t>
   </si>
   <si>
@@ -1002,9 +1026,6 @@
   </si>
   <si>
     <t xml:space="preserve"> @@@@</t>
-  </si>
-  <si>
-    <t>.@@@@</t>
   </si>
 </sst>
 </file>
@@ -2121,16 +2142,16 @@
         <v>9</v>
       </c>
       <c r="D47" t="s" s="0">
-        <v>117</v>
+        <v>10</v>
       </c>
       <c r="E47" t="s" s="0">
-        <v>118</v>
+        <v>11</v>
       </c>
       <c r="F47" t="s" s="0">
         <v>98</v>
       </c>
       <c r="G47" t="s" s="0">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="48">
@@ -2138,22 +2159,22 @@
         <v>115</v>
       </c>
       <c r="B48" t="s" s="0">
+        <v>118</v>
+      </c>
+      <c r="C48" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D48" t="s" s="0">
+        <v>119</v>
+      </c>
+      <c r="E48" t="s" s="0">
         <v>120</v>
-      </c>
-      <c r="C48" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D48" t="s" s="0">
-        <v>121</v>
-      </c>
-      <c r="E48" t="s" s="0">
-        <v>122</v>
       </c>
       <c r="F48" t="s" s="0">
         <v>98</v>
       </c>
       <c r="G48" t="s" s="0">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="49">
@@ -2161,16 +2182,16 @@
         <v>115</v>
       </c>
       <c r="B49" t="s" s="0">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C49" t="s" s="0">
         <v>33</v>
       </c>
       <c r="D49" t="s" s="0">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E49" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F49" t="s" s="0">
         <v>98</v>
@@ -2187,7 +2208,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K115"/>
+  <dimension ref="A1:K117"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -3534,7 +3555,7 @@
         <v>135</v>
       </c>
       <c r="E39" t="s" s="0">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F39" t="s" s="0">
         <v>135</v>
@@ -3569,7 +3590,7 @@
         <v>135</v>
       </c>
       <c r="E40" t="s" s="0">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F40" t="s" s="0">
         <v>135</v>
@@ -3581,7 +3602,7 @@
         <v>135</v>
       </c>
       <c r="I40" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="J40" t="s" s="0">
         <v>98</v>
@@ -3604,7 +3625,7 @@
         <v>135</v>
       </c>
       <c r="E41" t="s" s="0">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F41" t="s" s="0">
         <v>135</v>
@@ -3616,7 +3637,7 @@
         <v>135</v>
       </c>
       <c r="I41" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="J41" t="s" s="0">
         <v>98</v>
@@ -3741,7 +3762,7 @@
         <v>97</v>
       </c>
       <c r="D45" t="s" s="0">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E45" t="s" s="0">
         <v>10</v>
@@ -3776,7 +3797,7 @@
         <v>100</v>
       </c>
       <c r="D46" t="s" s="0">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E46" t="s" s="0">
         <v>10</v>
@@ -3788,7 +3809,7 @@
         <v>9</v>
       </c>
       <c r="H46" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I46" t="s" s="0">
         <v>11</v>
@@ -3811,7 +3832,7 @@
         <v>102</v>
       </c>
       <c r="D47" t="s" s="0">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E47" t="s" s="0">
         <v>10</v>
@@ -3823,7 +3844,7 @@
         <v>9</v>
       </c>
       <c r="H47" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I47" t="s" s="0">
         <v>11</v>
@@ -3849,7 +3870,7 @@
         <v>135</v>
       </c>
       <c r="E48" t="s" s="0">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F48" t="s" s="0">
         <v>135</v>
@@ -3884,7 +3905,7 @@
         <v>135</v>
       </c>
       <c r="E49" t="s" s="0">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F49" t="s" s="0">
         <v>135</v>
@@ -3896,7 +3917,7 @@
         <v>135</v>
       </c>
       <c r="I49" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="J49" t="s" s="0">
         <v>98</v>
@@ -3919,7 +3940,7 @@
         <v>135</v>
       </c>
       <c r="E50" t="s" s="0">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F50" t="s" s="0">
         <v>135</v>
@@ -3931,7 +3952,7 @@
         <v>135</v>
       </c>
       <c r="I50" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="J50" t="s" s="0">
         <v>98</v>
@@ -3954,7 +3975,7 @@
         <v>135</v>
       </c>
       <c r="E51" t="s" s="0">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F51" t="s" s="0">
         <v>135</v>
@@ -3966,7 +3987,7 @@
         <v>135</v>
       </c>
       <c r="I51" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="J51" t="s" s="0">
         <v>98</v>
@@ -3989,7 +4010,7 @@
         <v>135</v>
       </c>
       <c r="E52" t="s" s="0">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F52" t="s" s="0">
         <v>135</v>
@@ -4001,7 +4022,7 @@
         <v>135</v>
       </c>
       <c r="I52" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="J52" t="s" s="0">
         <v>98</v>
@@ -4021,7 +4042,7 @@
         <v>105</v>
       </c>
       <c r="D53" t="s" s="0">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E53" t="s" s="0">
         <v>10</v>
@@ -4056,7 +4077,7 @@
         <v>107</v>
       </c>
       <c r="D54" t="s" s="0">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E54" t="s" s="0">
         <v>10</v>
@@ -4068,7 +4089,7 @@
         <v>9</v>
       </c>
       <c r="H54" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I54" t="s" s="0">
         <v>11</v>
@@ -4091,10 +4112,10 @@
         <v>109</v>
       </c>
       <c r="D55" t="s" s="0">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E55" t="s" s="0">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F55" t="s" s="0">
         <v>9</v>
@@ -4103,7 +4124,7 @@
         <v>9</v>
       </c>
       <c r="H55" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I55" t="s" s="0">
         <v>195</v>
@@ -4126,10 +4147,10 @@
         <v>111</v>
       </c>
       <c r="D56" t="s" s="0">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E56" t="s" s="0">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F56" t="s" s="0">
         <v>9</v>
@@ -4138,7 +4159,7 @@
         <v>9</v>
       </c>
       <c r="H56" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I56" t="s" s="0">
         <v>197</v>
@@ -4161,7 +4182,7 @@
         <v>113</v>
       </c>
       <c r="D57" t="s" s="0">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E57" t="s" s="0">
         <v>10</v>
@@ -4173,7 +4194,7 @@
         <v>9</v>
       </c>
       <c r="H57" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I57" t="s" s="0">
         <v>11</v>
@@ -4196,10 +4217,10 @@
         <v>109</v>
       </c>
       <c r="D58" t="s" s="0">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E58" t="s" s="0">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F58" t="s" s="0">
         <v>9</v>
@@ -4231,7 +4252,7 @@
         <v>111</v>
       </c>
       <c r="D59" t="s" s="0">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E59" t="s" s="0">
         <v>10</v>
@@ -5806,10 +5827,10 @@
         <v>109</v>
       </c>
       <c r="D104" t="s" s="0">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E104" t="s" s="0">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F104" t="s" s="0">
         <v>9</v>
@@ -5911,7 +5932,7 @@
         <v>109</v>
       </c>
       <c r="D107" t="s" s="0">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E107" t="s" s="0">
         <v>10</v>
@@ -6124,7 +6145,7 @@
         <v>135</v>
       </c>
       <c r="E113" t="s" s="0">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F113" t="s" s="0">
         <v>135</v>
@@ -6136,13 +6157,13 @@
         <v>135</v>
       </c>
       <c r="I113" t="s" s="0">
-        <v>118</v>
+        <v>217</v>
       </c>
       <c r="J113" t="s" s="0">
         <v>98</v>
       </c>
       <c r="K113" t="s" s="0">
-        <v>119</v>
+        <v>218</v>
       </c>
     </row>
     <row r="114">
@@ -6153,13 +6174,13 @@
         <v>115</v>
       </c>
       <c r="C114" t="s" s="0">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D114" t="s" s="0">
         <v>135</v>
       </c>
       <c r="E114" t="s" s="0">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F114" t="s" s="0">
         <v>135</v>
@@ -6171,13 +6192,13 @@
         <v>135</v>
       </c>
       <c r="I114" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="J114" t="s" s="0">
         <v>98</v>
       </c>
       <c r="K114" t="s" s="0">
-        <v>123</v>
+        <v>219</v>
       </c>
     </row>
     <row r="115">
@@ -6188,13 +6209,13 @@
         <v>115</v>
       </c>
       <c r="C115" t="s" s="0">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D115" t="s" s="0">
         <v>135</v>
       </c>
       <c r="E115" t="s" s="0">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F115" t="s" s="0">
         <v>135</v>
@@ -6206,13 +6227,83 @@
         <v>135</v>
       </c>
       <c r="I115" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="J115" t="s" s="0">
         <v>98</v>
       </c>
       <c r="K115" t="s" s="0">
         <v>125</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="B116" t="s" s="0">
+        <v>115</v>
+      </c>
+      <c r="C116" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="D116" t="s" s="0">
+        <v>119</v>
+      </c>
+      <c r="E116" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F116" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="G116" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="H116" t="s" s="0">
+        <v>217</v>
+      </c>
+      <c r="I116" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="J116" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="K116" t="s" s="0">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="B117" t="s" s="0">
+        <v>115</v>
+      </c>
+      <c r="C117" t="s" s="0">
+        <v>118</v>
+      </c>
+      <c r="D117" t="s" s="0">
+        <v>123</v>
+      </c>
+      <c r="E117" t="s" s="0">
+        <v>119</v>
+      </c>
+      <c r="F117" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="G117" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="H117" t="s" s="0">
+        <v>124</v>
+      </c>
+      <c r="I117" t="s" s="0">
+        <v>120</v>
+      </c>
+      <c r="J117" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="K117" t="s" s="0">
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -6222,7 +6313,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J115"/>
+  <dimension ref="A1:J117"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -6236,7 +6327,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="E1" t="s" s="0">
         <v>126</v>
@@ -6245,16 +6336,16 @@
         <v>4</v>
       </c>
       <c r="G1" t="s" s="0">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="H1" t="s" s="0">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="I1" t="s" s="0">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="J1" t="s" s="0">
-        <v>221</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2">
@@ -6268,7 +6359,7 @@
         <v>9</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E2" t="s" s="0">
         <v>12</v>
@@ -6283,7 +6374,7 @@
         <v>11</v>
       </c>
       <c r="I2" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="3">
@@ -6297,7 +6388,7 @@
         <v>9</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E3" t="s" s="0">
         <v>12</v>
@@ -6312,7 +6403,7 @@
         <v>11</v>
       </c>
       <c r="I3" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="4">
@@ -6326,7 +6417,7 @@
         <v>9</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E4" t="s" s="0">
         <v>17</v>
@@ -6341,7 +6432,7 @@
         <v>11</v>
       </c>
       <c r="I4" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="5">
@@ -6355,7 +6446,7 @@
         <v>9</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E5" t="s" s="0">
         <v>20</v>
@@ -6370,7 +6461,7 @@
         <v>11</v>
       </c>
       <c r="I5" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="6">
@@ -6384,7 +6475,7 @@
         <v>9</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E6" t="s" s="0">
         <v>17</v>
@@ -6399,7 +6490,7 @@
         <v>11</v>
       </c>
       <c r="I6" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="7">
@@ -6413,7 +6504,7 @@
         <v>9</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E7" t="s" s="0">
         <v>17</v>
@@ -6428,7 +6519,7 @@
         <v>11</v>
       </c>
       <c r="I7" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="8">
@@ -6442,7 +6533,7 @@
         <v>9</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E8" t="s" s="0">
         <v>17</v>
@@ -6457,7 +6548,7 @@
         <v>11</v>
       </c>
       <c r="I8" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="9">
@@ -6471,7 +6562,7 @@
         <v>9</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E9" t="s" s="0">
         <v>20</v>
@@ -6486,7 +6577,7 @@
         <v>11</v>
       </c>
       <c r="I9" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="10">
@@ -6500,7 +6591,7 @@
         <v>33</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E10" t="s" s="0">
         <v>17</v>
@@ -6515,7 +6606,7 @@
         <v>11</v>
       </c>
       <c r="I10" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="11">
@@ -6529,7 +6620,7 @@
         <v>33</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E11" t="s" s="0">
         <v>12</v>
@@ -6544,7 +6635,7 @@
         <v>11</v>
       </c>
       <c r="I11" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="12">
@@ -6558,7 +6649,7 @@
         <v>33</v>
       </c>
       <c r="D12" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E12" t="s" s="0">
         <v>17</v>
@@ -6573,7 +6664,7 @@
         <v>11</v>
       </c>
       <c r="I12" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="13">
@@ -6587,7 +6678,7 @@
         <v>33</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E13" t="s" s="0">
         <v>12</v>
@@ -6602,7 +6693,7 @@
         <v>11</v>
       </c>
       <c r="I13" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="14">
@@ -6616,7 +6707,7 @@
         <v>33</v>
       </c>
       <c r="D14" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E14" t="s" s="0">
         <v>12</v>
@@ -6631,7 +6722,7 @@
         <v>11</v>
       </c>
       <c r="I14" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="15">
@@ -6645,7 +6736,7 @@
         <v>33</v>
       </c>
       <c r="D15" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E15" t="s" s="0">
         <v>20</v>
@@ -6660,7 +6751,7 @@
         <v>11</v>
       </c>
       <c r="I15" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="16">
@@ -6674,7 +6765,7 @@
         <v>33</v>
       </c>
       <c r="D16" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E16" t="s" s="0">
         <v>17</v>
@@ -6689,7 +6780,7 @@
         <v>11</v>
       </c>
       <c r="I16" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="17">
@@ -6703,7 +6794,7 @@
         <v>33</v>
       </c>
       <c r="D17" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E17" t="s" s="0">
         <v>17</v>
@@ -6718,7 +6809,7 @@
         <v>11</v>
       </c>
       <c r="I17" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="18">
@@ -6732,7 +6823,7 @@
         <v>33</v>
       </c>
       <c r="D18" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E18" t="s" s="0">
         <v>12</v>
@@ -6747,7 +6838,7 @@
         <v>11</v>
       </c>
       <c r="I18" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="19">
@@ -6761,7 +6852,7 @@
         <v>9</v>
       </c>
       <c r="D19" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E19" t="s" s="0">
         <v>12</v>
@@ -6776,7 +6867,7 @@
         <v>11</v>
       </c>
       <c r="I19" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="20">
@@ -6790,7 +6881,7 @@
         <v>9</v>
       </c>
       <c r="D20" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E20" t="s" s="0">
         <v>12</v>
@@ -6805,7 +6896,7 @@
         <v>11</v>
       </c>
       <c r="I20" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="21">
@@ -6819,7 +6910,7 @@
         <v>9</v>
       </c>
       <c r="D21" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E21" t="s" s="0">
         <v>20</v>
@@ -6834,7 +6925,7 @@
         <v>11</v>
       </c>
       <c r="I21" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="22">
@@ -6848,7 +6939,7 @@
         <v>9</v>
       </c>
       <c r="D22" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E22" t="s" s="0">
         <v>17</v>
@@ -6863,7 +6954,7 @@
         <v>11</v>
       </c>
       <c r="I22" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="23">
@@ -6877,7 +6968,7 @@
         <v>9</v>
       </c>
       <c r="D23" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E23" t="s" s="0">
         <v>12</v>
@@ -6892,7 +6983,7 @@
         <v>11</v>
       </c>
       <c r="I23" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="24">
@@ -6906,7 +6997,7 @@
         <v>9</v>
       </c>
       <c r="D24" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E24" t="s" s="0">
         <v>12</v>
@@ -6921,7 +7012,7 @@
         <v>11</v>
       </c>
       <c r="I24" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="25">
@@ -6935,7 +7026,7 @@
         <v>9</v>
       </c>
       <c r="D25" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E25" t="s" s="0">
         <v>12</v>
@@ -6950,7 +7041,7 @@
         <v>11</v>
       </c>
       <c r="I25" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="26">
@@ -6964,7 +7055,7 @@
         <v>9</v>
       </c>
       <c r="D26" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E26" t="s" s="0">
         <v>12</v>
@@ -6979,7 +7070,7 @@
         <v>11</v>
       </c>
       <c r="I26" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="27">
@@ -6993,7 +7084,7 @@
         <v>9</v>
       </c>
       <c r="D27" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E27" t="s" s="0">
         <v>12</v>
@@ -7008,7 +7099,7 @@
         <v>11</v>
       </c>
       <c r="I27" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="28">
@@ -7022,7 +7113,7 @@
         <v>9</v>
       </c>
       <c r="D28" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E28" t="s" s="0">
         <v>17</v>
@@ -7037,7 +7128,7 @@
         <v>11</v>
       </c>
       <c r="I28" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="29">
@@ -7051,7 +7142,7 @@
         <v>9</v>
       </c>
       <c r="D29" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E29" t="s" s="0">
         <v>17</v>
@@ -7066,7 +7157,7 @@
         <v>11</v>
       </c>
       <c r="I29" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="30">
@@ -7080,7 +7171,7 @@
         <v>9</v>
       </c>
       <c r="D30" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E30" t="s" s="0">
         <v>17</v>
@@ -7095,7 +7186,7 @@
         <v>11</v>
       </c>
       <c r="I30" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="31">
@@ -7109,7 +7200,7 @@
         <v>9</v>
       </c>
       <c r="D31" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E31" t="s" s="0">
         <v>17</v>
@@ -7124,7 +7215,7 @@
         <v>11</v>
       </c>
       <c r="I31" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="32">
@@ -7138,7 +7229,7 @@
         <v>9</v>
       </c>
       <c r="D32" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E32" t="s" s="0">
         <v>17</v>
@@ -7153,7 +7244,7 @@
         <v>11</v>
       </c>
       <c r="I32" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="33">
@@ -7167,7 +7258,7 @@
         <v>9</v>
       </c>
       <c r="D33" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E33" t="s" s="0">
         <v>17</v>
@@ -7182,7 +7273,7 @@
         <v>11</v>
       </c>
       <c r="I33" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="34">
@@ -7196,7 +7287,7 @@
         <v>9</v>
       </c>
       <c r="D34" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E34" t="s" s="0">
         <v>17</v>
@@ -7211,7 +7302,7 @@
         <v>11</v>
       </c>
       <c r="I34" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="35">
@@ -7225,7 +7316,7 @@
         <v>9</v>
       </c>
       <c r="D35" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E35" t="s" s="0">
         <v>17</v>
@@ -7240,7 +7331,7 @@
         <v>11</v>
       </c>
       <c r="I35" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="36">
@@ -7254,7 +7345,7 @@
         <v>9</v>
       </c>
       <c r="D36" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E36" t="s" s="0">
         <v>17</v>
@@ -7269,7 +7360,7 @@
         <v>11</v>
       </c>
       <c r="I36" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="37">
@@ -7283,7 +7374,7 @@
         <v>9</v>
       </c>
       <c r="D37" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E37" t="s" s="0">
         <v>17</v>
@@ -7298,7 +7389,7 @@
         <v>11</v>
       </c>
       <c r="I37" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="38">
@@ -7312,7 +7403,7 @@
         <v>9</v>
       </c>
       <c r="D38" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E38" t="s" s="0">
         <v>17</v>
@@ -7327,7 +7418,7 @@
         <v>11</v>
       </c>
       <c r="I38" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="39">
@@ -7341,7 +7432,7 @@
         <v>9</v>
       </c>
       <c r="D39" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E39" t="s" s="0">
         <v>98</v>
@@ -7356,7 +7447,7 @@
         <v>174</v>
       </c>
       <c r="I39" t="s" s="0">
-        <v>224</v>
+        <v>228</v>
       </c>
     </row>
     <row r="40">
@@ -7370,22 +7461,22 @@
         <v>9</v>
       </c>
       <c r="D40" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E40" t="s" s="0">
         <v>98</v>
       </c>
       <c r="F40" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G40" t="s" s="0">
         <v>135</v>
       </c>
       <c r="H40" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I40" t="s" s="0">
-        <v>225</v>
+        <v>229</v>
       </c>
     </row>
     <row r="41">
@@ -7399,22 +7490,22 @@
         <v>9</v>
       </c>
       <c r="D41" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E41" t="s" s="0">
         <v>98</v>
       </c>
       <c r="F41" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G41" t="s" s="0">
         <v>135</v>
       </c>
       <c r="H41" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I41" t="s" s="0">
-        <v>225</v>
+        <v>229</v>
       </c>
     </row>
     <row r="42">
@@ -7428,7 +7519,7 @@
         <v>9</v>
       </c>
       <c r="D42" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E42" t="s" s="0">
         <v>12</v>
@@ -7437,13 +7528,13 @@
         <v>11</v>
       </c>
       <c r="G42" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H42" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I42" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="43">
@@ -7457,7 +7548,7 @@
         <v>9</v>
       </c>
       <c r="D43" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E43" t="s" s="0">
         <v>12</v>
@@ -7466,13 +7557,13 @@
         <v>11</v>
       </c>
       <c r="G43" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H43" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I43" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="44">
@@ -7486,7 +7577,7 @@
         <v>9</v>
       </c>
       <c r="D44" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E44" t="s" s="0">
         <v>17</v>
@@ -7495,13 +7586,13 @@
         <v>11</v>
       </c>
       <c r="G44" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H44" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I44" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="45">
@@ -7515,7 +7606,7 @@
         <v>9</v>
       </c>
       <c r="D45" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E45" t="s" s="0">
         <v>98</v>
@@ -7524,13 +7615,13 @@
         <v>11</v>
       </c>
       <c r="G45" t="s" s="0">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="H45" t="s" s="0">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="I45" t="s" s="0">
-        <v>231</v>
+        <v>235</v>
       </c>
     </row>
     <row r="46">
@@ -7544,7 +7635,7 @@
         <v>9</v>
       </c>
       <c r="D46" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E46" t="s" s="0">
         <v>98</v>
@@ -7556,10 +7647,10 @@
         <v>11</v>
       </c>
       <c r="H46" t="s" s="0">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="I46" t="s" s="0">
-        <v>233</v>
+        <v>237</v>
       </c>
     </row>
     <row r="47">
@@ -7573,7 +7664,7 @@
         <v>9</v>
       </c>
       <c r="D47" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E47" t="s" s="0">
         <v>98</v>
@@ -7585,10 +7676,10 @@
         <v>11</v>
       </c>
       <c r="H47" t="s" s="0">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="I47" t="s" s="0">
-        <v>233</v>
+        <v>237</v>
       </c>
     </row>
     <row r="48">
@@ -7602,7 +7693,7 @@
         <v>9</v>
       </c>
       <c r="D48" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E48" t="s" s="0">
         <v>98</v>
@@ -7617,7 +7708,7 @@
         <v>186</v>
       </c>
       <c r="I48" t="s" s="0">
-        <v>234</v>
+        <v>238</v>
       </c>
     </row>
     <row r="49">
@@ -7631,22 +7722,22 @@
         <v>9</v>
       </c>
       <c r="D49" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E49" t="s" s="0">
         <v>98</v>
       </c>
       <c r="F49" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G49" t="s" s="0">
         <v>135</v>
       </c>
       <c r="H49" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I49" t="s" s="0">
-        <v>225</v>
+        <v>229</v>
       </c>
     </row>
     <row r="50">
@@ -7660,22 +7751,22 @@
         <v>9</v>
       </c>
       <c r="D50" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E50" t="s" s="0">
         <v>98</v>
       </c>
       <c r="F50" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G50" t="s" s="0">
         <v>135</v>
       </c>
       <c r="H50" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I50" t="s" s="0">
-        <v>225</v>
+        <v>229</v>
       </c>
     </row>
     <row r="51">
@@ -7689,22 +7780,22 @@
         <v>9</v>
       </c>
       <c r="D51" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E51" t="s" s="0">
         <v>98</v>
       </c>
       <c r="F51" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G51" t="s" s="0">
         <v>135</v>
       </c>
       <c r="H51" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I51" t="s" s="0">
-        <v>225</v>
+        <v>229</v>
       </c>
     </row>
     <row r="52">
@@ -7718,22 +7809,22 @@
         <v>9</v>
       </c>
       <c r="D52" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E52" t="s" s="0">
         <v>98</v>
       </c>
       <c r="F52" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G52" t="s" s="0">
         <v>135</v>
       </c>
       <c r="H52" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I52" t="s" s="0">
-        <v>225</v>
+        <v>229</v>
       </c>
     </row>
     <row r="53">
@@ -7747,7 +7838,7 @@
         <v>9</v>
       </c>
       <c r="D53" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E53" t="s" s="0">
         <v>98</v>
@@ -7756,13 +7847,13 @@
         <v>11</v>
       </c>
       <c r="G53" t="s" s="0">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H53" t="s" s="0">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="I53" t="s" s="0">
-        <v>237</v>
+        <v>241</v>
       </c>
     </row>
     <row r="54">
@@ -7776,7 +7867,7 @@
         <v>9</v>
       </c>
       <c r="D54" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E54" t="s" s="0">
         <v>98</v>
@@ -7788,10 +7879,10 @@
         <v>11</v>
       </c>
       <c r="H54" t="s" s="0">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="I54" t="s" s="0">
-        <v>233</v>
+        <v>237</v>
       </c>
     </row>
     <row r="55">
@@ -7805,7 +7896,7 @@
         <v>9</v>
       </c>
       <c r="D55" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E55" t="s" s="0">
         <v>98</v>
@@ -7817,10 +7908,10 @@
         <v>195</v>
       </c>
       <c r="H55" t="s" s="0">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I55" t="s" s="0">
-        <v>239</v>
+        <v>243</v>
       </c>
     </row>
     <row r="56">
@@ -7834,7 +7925,7 @@
         <v>9</v>
       </c>
       <c r="D56" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E56" t="s" s="0">
         <v>98</v>
@@ -7846,10 +7937,10 @@
         <v>197</v>
       </c>
       <c r="H56" t="s" s="0">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="I56" t="s" s="0">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="57">
@@ -7863,7 +7954,7 @@
         <v>9</v>
       </c>
       <c r="D57" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E57" t="s" s="0">
         <v>98</v>
@@ -7875,10 +7966,10 @@
         <v>11</v>
       </c>
       <c r="H57" t="s" s="0">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="I57" t="s" s="0">
-        <v>233</v>
+        <v>237</v>
       </c>
     </row>
     <row r="58">
@@ -7892,7 +7983,7 @@
         <v>9</v>
       </c>
       <c r="D58" t="s" s="0">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="E58" t="s" s="0">
         <v>98</v>
@@ -7901,13 +7992,13 @@
         <v>174</v>
       </c>
       <c r="G58" t="s" s="0">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="H58" t="s" s="0">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="I58" t="s" s="0">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="59">
@@ -7921,7 +8012,7 @@
         <v>9</v>
       </c>
       <c r="D59" t="s" s="0">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="E59" t="s" s="0">
         <v>98</v>
@@ -7930,13 +8021,13 @@
         <v>11</v>
       </c>
       <c r="G59" t="s" s="0">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="H59" t="s" s="0">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="I59" t="s" s="0">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="60">
@@ -7950,7 +8041,7 @@
         <v>9</v>
       </c>
       <c r="D60" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E60" t="s" s="0">
         <v>12</v>
@@ -7959,13 +8050,13 @@
         <v>11</v>
       </c>
       <c r="G60" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H60" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I60" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="61">
@@ -7979,7 +8070,7 @@
         <v>9</v>
       </c>
       <c r="D61" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E61" t="s" s="0">
         <v>12</v>
@@ -7988,13 +8079,13 @@
         <v>11</v>
       </c>
       <c r="G61" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H61" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I61" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="62">
@@ -8008,7 +8099,7 @@
         <v>9</v>
       </c>
       <c r="D62" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E62" t="s" s="0">
         <v>17</v>
@@ -8017,13 +8108,13 @@
         <v>11</v>
       </c>
       <c r="G62" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H62" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I62" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="63">
@@ -8037,7 +8128,7 @@
         <v>9</v>
       </c>
       <c r="D63" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E63" t="s" s="0">
         <v>20</v>
@@ -8046,13 +8137,13 @@
         <v>11</v>
       </c>
       <c r="G63" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H63" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I63" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="64">
@@ -8066,7 +8157,7 @@
         <v>9</v>
       </c>
       <c r="D64" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E64" t="s" s="0">
         <v>17</v>
@@ -8075,13 +8166,13 @@
         <v>11</v>
       </c>
       <c r="G64" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H64" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I64" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="65">
@@ -8095,7 +8186,7 @@
         <v>9</v>
       </c>
       <c r="D65" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E65" t="s" s="0">
         <v>17</v>
@@ -8104,13 +8195,13 @@
         <v>11</v>
       </c>
       <c r="G65" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H65" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I65" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="66">
@@ -8124,7 +8215,7 @@
         <v>9</v>
       </c>
       <c r="D66" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E66" t="s" s="0">
         <v>17</v>
@@ -8133,13 +8224,13 @@
         <v>11</v>
       </c>
       <c r="G66" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H66" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I66" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="67">
@@ -8153,7 +8244,7 @@
         <v>9</v>
       </c>
       <c r="D67" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E67" t="s" s="0">
         <v>20</v>
@@ -8162,13 +8253,13 @@
         <v>11</v>
       </c>
       <c r="G67" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H67" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I67" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="68">
@@ -8182,7 +8273,7 @@
         <v>33</v>
       </c>
       <c r="D68" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E68" t="s" s="0">
         <v>17</v>
@@ -8191,13 +8282,13 @@
         <v>11</v>
       </c>
       <c r="G68" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H68" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I68" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="69">
@@ -8211,7 +8302,7 @@
         <v>33</v>
       </c>
       <c r="D69" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E69" t="s" s="0">
         <v>12</v>
@@ -8220,13 +8311,13 @@
         <v>11</v>
       </c>
       <c r="G69" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H69" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I69" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="70">
@@ -8240,7 +8331,7 @@
         <v>33</v>
       </c>
       <c r="D70" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E70" t="s" s="0">
         <v>17</v>
@@ -8249,13 +8340,13 @@
         <v>11</v>
       </c>
       <c r="G70" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H70" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I70" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="71">
@@ -8269,7 +8360,7 @@
         <v>33</v>
       </c>
       <c r="D71" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E71" t="s" s="0">
         <v>12</v>
@@ -8278,13 +8369,13 @@
         <v>11</v>
       </c>
       <c r="G71" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H71" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I71" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="72">
@@ -8298,7 +8389,7 @@
         <v>33</v>
       </c>
       <c r="D72" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E72" t="s" s="0">
         <v>12</v>
@@ -8307,13 +8398,13 @@
         <v>11</v>
       </c>
       <c r="G72" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H72" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I72" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="73">
@@ -8327,7 +8418,7 @@
         <v>33</v>
       </c>
       <c r="D73" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E73" t="s" s="0">
         <v>20</v>
@@ -8336,13 +8427,13 @@
         <v>11</v>
       </c>
       <c r="G73" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H73" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I73" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="74">
@@ -8356,7 +8447,7 @@
         <v>33</v>
       </c>
       <c r="D74" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E74" t="s" s="0">
         <v>17</v>
@@ -8365,13 +8456,13 @@
         <v>11</v>
       </c>
       <c r="G74" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H74" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I74" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="75">
@@ -8385,7 +8476,7 @@
         <v>33</v>
       </c>
       <c r="D75" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E75" t="s" s="0">
         <v>17</v>
@@ -8394,13 +8485,13 @@
         <v>11</v>
       </c>
       <c r="G75" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H75" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I75" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="76">
@@ -8414,7 +8505,7 @@
         <v>33</v>
       </c>
       <c r="D76" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E76" t="s" s="0">
         <v>12</v>
@@ -8423,13 +8514,13 @@
         <v>11</v>
       </c>
       <c r="G76" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H76" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I76" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="77">
@@ -8443,7 +8534,7 @@
         <v>9</v>
       </c>
       <c r="D77" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E77" t="s" s="0">
         <v>12</v>
@@ -8452,13 +8543,13 @@
         <v>11</v>
       </c>
       <c r="G77" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H77" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I77" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="78">
@@ -8472,7 +8563,7 @@
         <v>9</v>
       </c>
       <c r="D78" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E78" t="s" s="0">
         <v>12</v>
@@ -8481,13 +8572,13 @@
         <v>11</v>
       </c>
       <c r="G78" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H78" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I78" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="79">
@@ -8501,7 +8592,7 @@
         <v>9</v>
       </c>
       <c r="D79" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E79" t="s" s="0">
         <v>20</v>
@@ -8510,13 +8601,13 @@
         <v>11</v>
       </c>
       <c r="G79" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H79" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I79" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="80">
@@ -8530,7 +8621,7 @@
         <v>9</v>
       </c>
       <c r="D80" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E80" t="s" s="0">
         <v>17</v>
@@ -8539,13 +8630,13 @@
         <v>11</v>
       </c>
       <c r="G80" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H80" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I80" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="81">
@@ -8559,7 +8650,7 @@
         <v>9</v>
       </c>
       <c r="D81" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E81" t="s" s="0">
         <v>12</v>
@@ -8568,13 +8659,13 @@
         <v>11</v>
       </c>
       <c r="G81" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H81" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I81" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="82">
@@ -8588,7 +8679,7 @@
         <v>9</v>
       </c>
       <c r="D82" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E82" t="s" s="0">
         <v>12</v>
@@ -8597,13 +8688,13 @@
         <v>11</v>
       </c>
       <c r="G82" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H82" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I82" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="83">
@@ -8617,7 +8708,7 @@
         <v>9</v>
       </c>
       <c r="D83" t="s" s="0">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="E83" t="s" s="0">
         <v>12</v>
@@ -8626,13 +8717,13 @@
         <v>11</v>
       </c>
       <c r="G83" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H83" t="s" s="0">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="I83" t="s" s="0">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="84">
@@ -8646,7 +8737,7 @@
         <v>9</v>
       </c>
       <c r="D84" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E84" t="s" s="0">
         <v>12</v>
@@ -8655,13 +8746,13 @@
         <v>11</v>
       </c>
       <c r="G84" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H84" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I84" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="85">
@@ -8675,7 +8766,7 @@
         <v>9</v>
       </c>
       <c r="D85" t="s" s="0">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="E85" t="s" s="0">
         <v>12</v>
@@ -8684,13 +8775,13 @@
         <v>11</v>
       </c>
       <c r="G85" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H85" t="s" s="0">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="I85" t="s" s="0">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="86">
@@ -8704,7 +8795,7 @@
         <v>9</v>
       </c>
       <c r="D86" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E86" t="s" s="0">
         <v>17</v>
@@ -8713,13 +8804,13 @@
         <v>11</v>
       </c>
       <c r="G86" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H86" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I86" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="87">
@@ -8733,7 +8824,7 @@
         <v>9</v>
       </c>
       <c r="D87" t="s" s="0">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="E87" t="s" s="0">
         <v>17</v>
@@ -8742,13 +8833,13 @@
         <v>11</v>
       </c>
       <c r="G87" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H87" t="s" s="0">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="I87" t="s" s="0">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="88">
@@ -8762,7 +8853,7 @@
         <v>9</v>
       </c>
       <c r="D88" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E88" t="s" s="0">
         <v>17</v>
@@ -8771,13 +8862,13 @@
         <v>11</v>
       </c>
       <c r="G88" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H88" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I88" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="89">
@@ -8791,7 +8882,7 @@
         <v>9</v>
       </c>
       <c r="D89" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E89" t="s" s="0">
         <v>17</v>
@@ -8800,13 +8891,13 @@
         <v>11</v>
       </c>
       <c r="G89" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H89" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I89" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="90">
@@ -8820,7 +8911,7 @@
         <v>9</v>
       </c>
       <c r="D90" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E90" t="s" s="0">
         <v>17</v>
@@ -8829,13 +8920,13 @@
         <v>11</v>
       </c>
       <c r="G90" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H90" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I90" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="91">
@@ -8849,7 +8940,7 @@
         <v>9</v>
       </c>
       <c r="D91" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E91" t="s" s="0">
         <v>17</v>
@@ -8858,13 +8949,13 @@
         <v>11</v>
       </c>
       <c r="G91" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H91" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I91" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="92">
@@ -8878,7 +8969,7 @@
         <v>9</v>
       </c>
       <c r="D92" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E92" t="s" s="0">
         <v>17</v>
@@ -8887,13 +8978,13 @@
         <v>11</v>
       </c>
       <c r="G92" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H92" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I92" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="93">
@@ -8907,7 +8998,7 @@
         <v>9</v>
       </c>
       <c r="D93" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E93" t="s" s="0">
         <v>17</v>
@@ -8916,13 +9007,13 @@
         <v>11</v>
       </c>
       <c r="G93" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H93" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I93" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="94">
@@ -8936,7 +9027,7 @@
         <v>9</v>
       </c>
       <c r="D94" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E94" t="s" s="0">
         <v>17</v>
@@ -8945,13 +9036,13 @@
         <v>11</v>
       </c>
       <c r="G94" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H94" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I94" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="95">
@@ -8965,7 +9056,7 @@
         <v>9</v>
       </c>
       <c r="D95" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E95" t="s" s="0">
         <v>17</v>
@@ -8974,13 +9065,13 @@
         <v>11</v>
       </c>
       <c r="G95" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H95" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I95" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="96">
@@ -8994,7 +9085,7 @@
         <v>9</v>
       </c>
       <c r="D96" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E96" t="s" s="0">
         <v>17</v>
@@ -9003,13 +9094,13 @@
         <v>11</v>
       </c>
       <c r="G96" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H96" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="I96" t="s" s="0">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="97">
@@ -9023,7 +9114,7 @@
         <v>9</v>
       </c>
       <c r="D97" t="s" s="0">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="E97" t="s" s="0">
         <v>98</v>
@@ -9032,13 +9123,13 @@
         <v>11</v>
       </c>
       <c r="G97" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H97" t="s" s="0">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="I97" t="s" s="0">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="98">
@@ -9052,7 +9143,7 @@
         <v>9</v>
       </c>
       <c r="D98" t="s" s="0">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="E98" t="s" s="0">
         <v>98</v>
@@ -9061,13 +9152,13 @@
         <v>11</v>
       </c>
       <c r="G98" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H98" t="s" s="0">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="I98" t="s" s="0">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="99">
@@ -9081,7 +9172,7 @@
         <v>9</v>
       </c>
       <c r="D99" t="s" s="0">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="E99" t="s" s="0">
         <v>98</v>
@@ -9090,13 +9181,13 @@
         <v>11</v>
       </c>
       <c r="G99" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H99" t="s" s="0">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="I99" t="s" s="0">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="100">
@@ -9110,7 +9201,7 @@
         <v>9</v>
       </c>
       <c r="D100" t="s" s="0">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="E100" t="s" s="0">
         <v>98</v>
@@ -9119,13 +9210,13 @@
         <v>11</v>
       </c>
       <c r="G100" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H100" t="s" s="0">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="I100" t="s" s="0">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="101">
@@ -9139,7 +9230,7 @@
         <v>9</v>
       </c>
       <c r="D101" t="s" s="0">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="E101" t="s" s="0">
         <v>98</v>
@@ -9148,13 +9239,13 @@
         <v>11</v>
       </c>
       <c r="G101" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H101" t="s" s="0">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="I101" t="s" s="0">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="102">
@@ -9168,7 +9259,7 @@
         <v>9</v>
       </c>
       <c r="D102" t="s" s="0">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="E102" t="s" s="0">
         <v>98</v>
@@ -9177,13 +9268,13 @@
         <v>11</v>
       </c>
       <c r="G102" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H102" t="s" s="0">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="I102" t="s" s="0">
-        <v>259</v>
+        <v>263</v>
       </c>
     </row>
     <row r="103">
@@ -9197,7 +9288,7 @@
         <v>9</v>
       </c>
       <c r="D103" t="s" s="0">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="E103" t="s" s="0">
         <v>98</v>
@@ -9206,13 +9297,13 @@
         <v>11</v>
       </c>
       <c r="G103" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H103" t="s" s="0">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="I103" t="s" s="0">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="104">
@@ -9226,7 +9317,7 @@
         <v>9</v>
       </c>
       <c r="D104" t="s" s="0">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="E104" t="s" s="0">
         <v>98</v>
@@ -9235,13 +9326,13 @@
         <v>212</v>
       </c>
       <c r="G104" t="s" s="0">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="H104" t="s" s="0">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="I104" t="s" s="0">
-        <v>261</v>
+        <v>265</v>
       </c>
     </row>
     <row r="105">
@@ -9255,7 +9346,7 @@
         <v>9</v>
       </c>
       <c r="D105" t="s" s="0">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="E105" t="s" s="0">
         <v>98</v>
@@ -9264,13 +9355,13 @@
         <v>11</v>
       </c>
       <c r="G105" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H105" t="s" s="0">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="I105" t="s" s="0">
-        <v>263</v>
+        <v>267</v>
       </c>
     </row>
     <row r="106">
@@ -9284,7 +9375,7 @@
         <v>9</v>
       </c>
       <c r="D106" t="s" s="0">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="E106" t="s" s="0">
         <v>98</v>
@@ -9293,13 +9384,13 @@
         <v>11</v>
       </c>
       <c r="G106" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H106" t="s" s="0">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="I106" t="s" s="0">
-        <v>265</v>
+        <v>269</v>
       </c>
     </row>
     <row r="107">
@@ -9313,7 +9404,7 @@
         <v>9</v>
       </c>
       <c r="D107" t="s" s="0">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="E107" t="s" s="0">
         <v>98</v>
@@ -9322,13 +9413,13 @@
         <v>11</v>
       </c>
       <c r="G107" t="s" s="0">
-        <v>267</v>
+        <v>120</v>
       </c>
       <c r="H107" t="s" s="0">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="I107" t="s" s="0">
-        <v>269</v>
+        <v>272</v>
       </c>
     </row>
     <row r="108">
@@ -9342,7 +9433,7 @@
         <v>9</v>
       </c>
       <c r="D108" t="s" s="0">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="E108" t="s" s="0">
         <v>98</v>
@@ -9351,13 +9442,13 @@
         <v>11</v>
       </c>
       <c r="G108" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H108" t="s" s="0">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="I108" t="s" s="0">
-        <v>271</v>
+        <v>274</v>
       </c>
     </row>
     <row r="109">
@@ -9371,7 +9462,7 @@
         <v>9</v>
       </c>
       <c r="D109" t="s" s="0">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="E109" t="s" s="0">
         <v>98</v>
@@ -9380,13 +9471,13 @@
         <v>11</v>
       </c>
       <c r="G109" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H109" t="s" s="0">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="I109" t="s" s="0">
-        <v>265</v>
+        <v>269</v>
       </c>
     </row>
     <row r="110">
@@ -9400,7 +9491,7 @@
         <v>9</v>
       </c>
       <c r="D110" t="s" s="0">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="E110" t="s" s="0">
         <v>98</v>
@@ -9409,13 +9500,13 @@
         <v>11</v>
       </c>
       <c r="G110" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H110" t="s" s="0">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="I110" t="s" s="0">
-        <v>273</v>
+        <v>276</v>
       </c>
     </row>
     <row r="111">
@@ -9429,7 +9520,7 @@
         <v>9</v>
       </c>
       <c r="D111" t="s" s="0">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="E111" t="s" s="0">
         <v>98</v>
@@ -9438,13 +9529,13 @@
         <v>11</v>
       </c>
       <c r="G111" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H111" t="s" s="0">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="I111" t="s" s="0">
-        <v>265</v>
+        <v>269</v>
       </c>
     </row>
     <row r="112">
@@ -9458,7 +9549,7 @@
         <v>9</v>
       </c>
       <c r="D112" t="s" s="0">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="E112" t="s" s="0">
         <v>98</v>
@@ -9467,13 +9558,13 @@
         <v>11</v>
       </c>
       <c r="G112" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H112" t="s" s="0">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="I112" t="s" s="0">
-        <v>265</v>
+        <v>269</v>
       </c>
     </row>
     <row r="113">
@@ -9487,22 +9578,22 @@
         <v>9</v>
       </c>
       <c r="D113" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E113" t="s" s="0">
         <v>98</v>
       </c>
       <c r="F113" t="s" s="0">
-        <v>118</v>
+        <v>217</v>
       </c>
       <c r="G113" t="s" s="0">
         <v>135</v>
       </c>
       <c r="H113" t="s" s="0">
-        <v>118</v>
+        <v>217</v>
       </c>
       <c r="I113" t="s" s="0">
-        <v>234</v>
+        <v>238</v>
       </c>
     </row>
     <row r="114">
@@ -9510,28 +9601,28 @@
         <v>115</v>
       </c>
       <c r="B114" t="s" s="0">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C114" t="s" s="0">
         <v>9</v>
       </c>
       <c r="D114" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E114" t="s" s="0">
         <v>98</v>
       </c>
       <c r="F114" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G114" t="s" s="0">
         <v>135</v>
       </c>
       <c r="H114" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I114" t="s" s="0">
-        <v>225</v>
+        <v>229</v>
       </c>
     </row>
     <row r="115">
@@ -9539,28 +9630,86 @@
         <v>115</v>
       </c>
       <c r="B115" t="s" s="0">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C115" t="s" s="0">
         <v>33</v>
       </c>
       <c r="D115" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E115" t="s" s="0">
         <v>98</v>
       </c>
       <c r="F115" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G115" t="s" s="0">
         <v>135</v>
       </c>
       <c r="H115" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I115" t="s" s="0">
-        <v>225</v>
+        <v>229</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="s" s="0">
+        <v>115</v>
+      </c>
+      <c r="B116" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="C116" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D116" t="s" s="0">
+        <v>230</v>
+      </c>
+      <c r="E116" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="F116" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="G116" t="s" s="0">
+        <v>277</v>
+      </c>
+      <c r="H116" t="s" s="0">
+        <v>278</v>
+      </c>
+      <c r="I116" t="s" s="0">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="s" s="0">
+        <v>115</v>
+      </c>
+      <c r="B117" t="s" s="0">
+        <v>118</v>
+      </c>
+      <c r="C117" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D117" t="s" s="0">
+        <v>230</v>
+      </c>
+      <c r="E117" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="F117" t="s" s="0">
+        <v>120</v>
+      </c>
+      <c r="G117" t="s" s="0">
+        <v>120</v>
+      </c>
+      <c r="H117" t="s" s="0">
+        <v>279</v>
+      </c>
+      <c r="I117" t="s" s="0">
+        <v>280</v>
       </c>
     </row>
   </sheetData>
@@ -9575,165 +9724,165 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="E1" t="s" s="0">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="F1" t="s" s="0">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="G1" t="s" s="0">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="H1" t="s" s="0">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="I1" t="s" s="0">
-        <v>281</v>
+        <v>288</v>
       </c>
       <c r="J1" t="s" s="0">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="K1" t="s" s="0">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="L1" t="s" s="0">
-        <v>284</v>
+        <v>291</v>
       </c>
       <c r="M1" t="s" s="0">
-        <v>285</v>
+        <v>292</v>
       </c>
       <c r="N1" t="s" s="0">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="O1" t="s" s="0">
-        <v>287</v>
+        <v>294</v>
       </c>
       <c r="P1" t="s" s="0">
-        <v>288</v>
+        <v>295</v>
       </c>
       <c r="Q1" t="s" s="0">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="R1" t="s" s="0">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="S1" t="s" s="0">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="T1" t="s" s="0">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="U1" t="s" s="0">
-        <v>293</v>
+        <v>300</v>
       </c>
       <c r="V1" t="s" s="0">
-        <v>294</v>
+        <v>301</v>
       </c>
       <c r="W1" t="s" s="0">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="X1" t="s" s="0">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="Y1" t="s" s="0">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="Z1" t="s" s="0">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="AA1" t="s" s="0">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="AB1" t="s" s="0">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="AC1" t="s" s="0">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="AD1" t="s" s="0">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="AE1" t="s" s="0">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="AF1" t="s" s="0">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="AG1" t="s" s="0">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="AH1" t="s" s="0">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="AI1" t="s" s="0">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="AJ1" t="s" s="0">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="AK1" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="AL1" t="s" s="0">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="AM1" t="s" s="0">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="AN1" t="s" s="0">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="AO1" t="s" s="0">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="AP1" t="s" s="0">
-        <v>314</v>
+        <v>321</v>
       </c>
       <c r="AQ1" t="s" s="0">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="AR1" t="s" s="0">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="AS1" t="s" s="0">
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="AT1" t="s" s="0">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="AU1" t="s" s="0">
-        <v>319</v>
+        <v>326</v>
       </c>
       <c r="AV1" t="s" s="0">
-        <v>320</v>
+        <v>327</v>
       </c>
       <c r="AW1" t="s" s="0">
-        <v>321</v>
+        <v>328</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>118</v>
+        <v>217</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E2" t="s" s="0">
         <v>11</v>
@@ -9850,22 +9999,22 @@
         <v>174</v>
       </c>
       <c r="AQ2" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AR2" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AS2" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AT2" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AU2" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AV2" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AW2" t="s" s="0">
         <v>186</v>
@@ -9873,13 +10022,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>135</v>
+        <v>120</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>135</v>
+        <v>11</v>
       </c>
       <c r="D3" t="s" s="0">
         <v>135</v>
@@ -10022,7 +10171,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B4" t="s" s="0">
         <v>135</v>
@@ -10171,7 +10320,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="B5" t="s" s="0">
         <v>135</v>
@@ -10320,7 +10469,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="B6" t="s" s="0">
         <v>135</v>
@@ -10472,51 +10621,51 @@
         <v>1</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>322</v>
+        <v>329</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="C10" t="s" s="0">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>324</v>
+        <v>331</v>
       </c>
       <c r="C11" t="s" s="0">
-        <v>118</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>323</v>
+        <v>332</v>
       </c>
       <c r="C12" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C13" t="s" s="0">
         <v>11</v>
@@ -10524,10 +10673,10 @@
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C14" t="s" s="0">
         <v>11</v>
@@ -10535,10 +10684,10 @@
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C15" t="s" s="0">
         <v>11</v>
@@ -10546,10 +10695,10 @@
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C16" t="s" s="0">
         <v>11</v>
@@ -10557,10 +10706,10 @@
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>281</v>
+        <v>288</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C17" t="s" s="0">
         <v>11</v>
@@ -10568,10 +10717,10 @@
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C18" t="s" s="0">
         <v>11</v>
@@ -10579,10 +10728,10 @@
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C19" t="s" s="0">
         <v>11</v>
@@ -10590,10 +10739,10 @@
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>284</v>
+        <v>291</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C20" t="s" s="0">
         <v>11</v>
@@ -10601,10 +10750,10 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>285</v>
+        <v>292</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C21" t="s" s="0">
         <v>11</v>
@@ -10612,10 +10761,10 @@
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C22" t="s" s="0">
         <v>11</v>
@@ -10623,10 +10772,10 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>287</v>
+        <v>294</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C23" t="s" s="0">
         <v>11</v>
@@ -10634,10 +10783,10 @@
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>288</v>
+        <v>295</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C24" t="s" s="0">
         <v>11</v>
@@ -10645,10 +10794,10 @@
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C25" t="s" s="0">
         <v>11</v>
@@ -10656,10 +10805,10 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C26" t="s" s="0">
         <v>11</v>
@@ -10667,10 +10816,10 @@
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B27" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C27" t="s" s="0">
         <v>11</v>
@@ -10678,10 +10827,10 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C28" t="s" s="0">
         <v>11</v>
@@ -10689,10 +10838,10 @@
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>293</v>
+        <v>300</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C29" t="s" s="0">
         <v>11</v>
@@ -10700,10 +10849,10 @@
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>294</v>
+        <v>301</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C30" t="s" s="0">
         <v>11</v>
@@ -10711,10 +10860,10 @@
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="B31" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C31" t="s" s="0">
         <v>11</v>
@@ -10722,10 +10871,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="B32" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C32" t="s" s="0">
         <v>11</v>
@@ -10733,10 +10882,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="B33" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C33" t="s" s="0">
         <v>11</v>
@@ -10744,10 +10893,10 @@
     </row>
     <row r="34">
       <c r="A34" t="s" s="0">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="B34" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C34" t="s" s="0">
         <v>11</v>
@@ -10755,10 +10904,10 @@
     </row>
     <row r="35">
       <c r="A35" t="s" s="0">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="B35" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C35" t="s" s="0">
         <v>11</v>
@@ -10766,10 +10915,10 @@
     </row>
     <row r="36">
       <c r="A36" t="s" s="0">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="B36" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C36" t="s" s="0">
         <v>11</v>
@@ -10777,10 +10926,10 @@
     </row>
     <row r="37">
       <c r="A37" t="s" s="0">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="B37" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C37" t="s" s="0">
         <v>11</v>
@@ -10788,10 +10937,10 @@
     </row>
     <row r="38">
       <c r="A38" t="s" s="0">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="B38" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C38" t="s" s="0">
         <v>11</v>
@@ -10799,10 +10948,10 @@
     </row>
     <row r="39">
       <c r="A39" t="s" s="0">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="B39" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C39" t="s" s="0">
         <v>11</v>
@@ -10810,10 +10959,10 @@
     </row>
     <row r="40">
       <c r="A40" t="s" s="0">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="B40" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C40" t="s" s="0">
         <v>11</v>
@@ -10821,10 +10970,10 @@
     </row>
     <row r="41">
       <c r="A41" t="s" s="0">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="B41" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C41" t="s" s="0">
         <v>11</v>
@@ -10832,10 +10981,10 @@
     </row>
     <row r="42">
       <c r="A42" t="s" s="0">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="B42" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C42" t="s" s="0">
         <v>11</v>
@@ -10843,10 +10992,10 @@
     </row>
     <row r="43">
       <c r="A43" t="s" s="0">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="B43" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C43" t="s" s="0">
         <v>11</v>
@@ -10854,10 +11003,10 @@
     </row>
     <row r="44">
       <c r="A44" t="s" s="0">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="B44" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C44" t="s" s="0">
         <v>11</v>
@@ -10865,10 +11014,10 @@
     </row>
     <row r="45">
       <c r="A45" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="B45" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C45" t="s" s="0">
         <v>11</v>
@@ -10876,10 +11025,10 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="0">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="B46" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C46" t="s" s="0">
         <v>11</v>
@@ -10887,10 +11036,10 @@
     </row>
     <row r="47">
       <c r="A47" t="s" s="0">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="B47" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C47" t="s" s="0">
         <v>11</v>
@@ -10898,10 +11047,10 @@
     </row>
     <row r="48">
       <c r="A48" t="s" s="0">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="B48" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C48" t="s" s="0">
         <v>11</v>
@@ -10909,10 +11058,10 @@
     </row>
     <row r="49">
       <c r="A49" t="s" s="0">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="B49" t="s" s="0">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C49" t="s" s="0">
         <v>11</v>
@@ -10920,10 +11069,10 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="0">
-        <v>314</v>
+        <v>321</v>
       </c>
       <c r="B50" t="s" s="0">
-        <v>326</v>
+        <v>334</v>
       </c>
       <c r="C50" t="s" s="0">
         <v>11</v>
@@ -10931,10 +11080,10 @@
     </row>
     <row r="51">
       <c r="A51" t="s" s="0">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="B51" t="s" s="0">
-        <v>327</v>
+        <v>335</v>
       </c>
       <c r="C51" t="s" s="0">
         <v>11</v>
@@ -10942,10 +11091,10 @@
     </row>
     <row r="52">
       <c r="A52" t="s" s="0">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="B52" t="s" s="0">
-        <v>327</v>
+        <v>335</v>
       </c>
       <c r="C52" t="s" s="0">
         <v>11</v>
@@ -10953,10 +11102,10 @@
     </row>
     <row r="53">
       <c r="A53" t="s" s="0">
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="B53" t="s" s="0">
-        <v>327</v>
+        <v>335</v>
       </c>
       <c r="C53" t="s" s="0">
         <v>11</v>
@@ -10964,10 +11113,10 @@
     </row>
     <row r="54">
       <c r="A54" t="s" s="0">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="B54" t="s" s="0">
-        <v>327</v>
+        <v>335</v>
       </c>
       <c r="C54" t="s" s="0">
         <v>11</v>
@@ -10975,10 +11124,10 @@
     </row>
     <row r="55">
       <c r="A55" t="s" s="0">
-        <v>319</v>
+        <v>326</v>
       </c>
       <c r="B55" t="s" s="0">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="C55" t="s" s="0">
         <v>11</v>
@@ -10986,10 +11135,10 @@
     </row>
     <row r="56">
       <c r="A56" t="s" s="0">
-        <v>320</v>
+        <v>327</v>
       </c>
       <c r="B56" t="s" s="0">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="C56" t="s" s="0">
         <v>11</v>
@@ -10997,10 +11146,10 @@
     </row>
     <row r="57">
       <c r="A57" t="s" s="0">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="B57" t="s" s="0">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="C57" t="s" s="0">
         <v>11</v>

</xml_diff>